<commit_message>
Model brochure-backed project content
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf1d42a66d66340e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rd9d6236e94134c71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R49b41ff48296475b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R3e4342d75c0b4ff6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Re4f225e477074bab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rbe7fad4f1a984016"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re07339e2ea1e49c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R04c64ce6f7fc4cef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R6a02233377cd42d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Re80f076b9fa646b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rbff9d76a2e694552"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R30982225fc98455e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,7 +22,7 @@
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="22">
+  <x:fonts count="23">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -147,8 +147,14 @@
       <x:color rgb="FF1F5C4A"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF17233D"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -183,6 +189,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFC89B3C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCE6F1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCE6F1"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -272,7 +288,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="173">
+  <x:cellXfs count="180">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -698,6 +714,27 @@
     <x:xf numFmtId="201" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="22" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -709,7 +746,7 @@
         <x:color rgb="FF374151"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5E7EB"/>
         </x:patternFill>
       </x:fill>
@@ -720,7 +757,7 @@
         <x:color rgb="FF1E40AF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -731,7 +768,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -742,7 +779,7 @@
         <x:color rgb="FF6B21A8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF3E8FF"/>
         </x:patternFill>
       </x:fill>
@@ -753,7 +790,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -764,7 +801,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -775,7 +812,7 @@
         <x:color rgb="FF374151"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5E7EB"/>
         </x:patternFill>
       </x:fill>
@@ -786,7 +823,7 @@
         <x:color rgb="FF1E40AF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -797,7 +834,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -808,7 +845,7 @@
         <x:color rgb="FF6B21A8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF3E8FF"/>
         </x:patternFill>
       </x:fill>
@@ -819,7 +856,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -830,7 +867,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -841,7 +878,7 @@
         <x:color rgb="FF374151"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5E7EB"/>
         </x:patternFill>
       </x:fill>
@@ -852,7 +889,7 @@
         <x:color rgb="FF1E40AF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -863,7 +900,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -874,7 +911,7 @@
         <x:color rgb="FF6B21A8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF3E8FF"/>
         </x:patternFill>
       </x:fill>
@@ -885,7 +922,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -896,7 +933,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -907,7 +944,7 @@
         <x:color rgb="FF374151"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5E7EB"/>
         </x:patternFill>
       </x:fill>
@@ -918,7 +955,7 @@
         <x:color rgb="FF1E40AF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -929,7 +966,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -940,7 +977,7 @@
         <x:color rgb="FF6B21A8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF3E8FF"/>
         </x:patternFill>
       </x:fill>
@@ -951,7 +988,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -962,7 +999,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -973,7 +1010,7 @@
         <x:color rgb="FF374151"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5E7EB"/>
         </x:patternFill>
       </x:fill>
@@ -984,7 +1021,7 @@
         <x:color rgb="FF1E40AF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDBEAFE"/>
         </x:patternFill>
       </x:fill>
@@ -995,7 +1032,7 @@
         <x:color rgb="FF92400E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEF3C7"/>
         </x:patternFill>
       </x:fill>
@@ -1006,7 +1043,7 @@
         <x:color rgb="FF6B21A8"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF3E8FF"/>
         </x:patternFill>
       </x:fill>
@@ -1017,7 +1054,7 @@
         <x:color rgb="FF166534"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDCFCE7"/>
         </x:patternFill>
       </x:fill>
@@ -1028,7 +1065,7 @@
         <x:color rgb="FF991B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFEE2E2"/>
         </x:patternFill>
       </x:fill>
@@ -1084,7 +1121,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReviewGuidelines" displayName="ReviewGuidelines" ref="A5:G34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ReviewGuidelines" displayName="ReviewGuidelines" ref="A5:G35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Guideline ID"/>
     <x:tableColumn id="2" name="Area"/>
@@ -1338,7 +1375,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="121" t="str">
-        <x:v>Accelerated evidence-led delivery plan targeting a production release by 30 December 2026.</x:v>
+        <x:v>Production plan resumed on 3 October 2026. The preserved Glitz Pride mockup is the approved UI reference; production release remains targeted for 30 December 2026.</x:v>
       </x:c>
       <x:c r="B2" s="120"/>
       <x:c r="C2" s="120"/>
@@ -1425,7 +1462,6 @@
         <x:v>Total tasks</x:v>
       </x:c>
       <x:c r="B7" s="127" t="n">
-        <x:f>COUNTA('Phase 1 MVP'!B6:B33)+COUNTA('Phase 2 MVP'!B6:B30)</x:f>
         <x:v>53</x:v>
       </x:c>
       <x:c r="C7" s="120"/>
@@ -1433,13 +1469,13 @@
         <x:v>Phase 1</x:v>
       </x:c>
       <x:c r="E7" s="128" t="str">
-        <x:v>Responsive property website with approved content and conversion journeys</x:v>
+        <x:v>Responsive property website using the preserved mockup UI, approved content, and production conversion journeys</x:v>
       </x:c>
       <x:c r="F7" s="129" t="n">
         <x:v>46267</x:v>
       </x:c>
       <x:c r="G7" s="129" t="n">
-        <x:v>46325</x:v>
+        <x:v>46351</x:v>
       </x:c>
       <x:c r="H7" s="128" t="n">
         <x:v>28</x:v>
@@ -1448,7 +1484,7 @@
         <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J7" s="128" t="str">
-        <x:v>Responsive QA, E2E tests, accessibility, performance, and UAT accepted</x:v>
+        <x:v>Mockup-to-production UI acceptance, responsive QA, E2E tests, accessibility, performance, and UAT accepted</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="52" customHeight="1">
@@ -1456,8 +1492,7 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="B8" s="131" t="n">
-        <x:f>COUNTIF('Phase 1 MVP'!I6:I33,"Completed")+COUNTIF('Phase 2 MVP'!I6:I30,"Completed")</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C8" s="120"/>
       <x:c r="D8" s="132" t="str">
@@ -1467,7 +1502,7 @@
         <x:v>Grounded AI concierge with dynamic previews, citations, recommendations, and handoff</x:v>
       </x:c>
       <x:c r="F8" s="133" t="n">
-        <x:v>46321</x:v>
+        <x:v>46342</x:v>
       </x:c>
       <x:c r="G8" s="133" t="n">
         <x:v>46386</x:v>
@@ -1487,7 +1522,6 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B9" s="131" t="n">
-        <x:f>COUNTIF('Phase 1 MVP'!I6:I33,"Planned")+COUNTIF('Phase 2 MVP'!I6:I30,"Planned")</x:f>
         <x:v>20</x:v>
       </x:c>
       <x:c r="C9" s="120"/>
@@ -1504,7 +1538,6 @@
         <x:v>Not started</x:v>
       </x:c>
       <x:c r="B10" s="131" t="n">
-        <x:f>COUNTIF('Phase 1 MVP'!I6:I33,"Not Started")+COUNTIF('Phase 2 MVP'!I6:I30,"Not Started")</x:f>
         <x:v>25</x:v>
       </x:c>
       <x:c r="C10" s="120"/>
@@ -1521,8 +1554,7 @@
         <x:v>In progress</x:v>
       </x:c>
       <x:c r="B11" s="131" t="n">
-        <x:f>COUNTIF('Phase 1 MVP'!I6:I33,"In Progress")+COUNTIF('Phase 2 MVP'!I6:I30,"In Progress")</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C11" s="120"/>
       <x:c r="D11" s="120"/>
@@ -1538,8 +1570,7 @@
         <x:v>Blocked / On hold</x:v>
       </x:c>
       <x:c r="B12" s="135" t="n">
-        <x:f>COUNTIF('Phase 1 MVP'!I6:I33,"Blocked")+COUNTIF('Phase 2 MVP'!I6:I30,"Blocked")+COUNTIF('Phase 1 MVP'!I6:I33,"On Hold")+COUNTIF('Phase 2 MVP'!I6:I30,"On Hold")</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C12" s="120"/>
       <x:c r="D12" s="120"/>
@@ -1772,16 +1803,16 @@
     </x:row>
     <x:row r="27" ht="42" customHeight="1">
       <x:c r="A27" s="128" t="str">
-        <x:v>Foundation and design system</x:v>
+        <x:v>Design baseline and content model</x:v>
       </x:c>
       <x:c r="B27" s="129" t="n">
-        <x:v>46295</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="C27" s="128" t="str">
-        <x:v>Approved design tokens, responsive shell, and core architecture</x:v>
+        <x:v>Preserved mockup reference, approved design tokens, and validated evidence-aware project content schema</x:v>
       </x:c>
       <x:c r="D27" s="128" t="str">
-        <x:v>Weekly working increments</x:v>
+        <x:v>Completed; mockup files remain unchanged</x:v>
       </x:c>
       <x:c r="E27" s="120"/>
       <x:c r="F27" s="120"/>
@@ -1795,13 +1826,13 @@
         <x:v>Phase 1 feature complete</x:v>
       </x:c>
       <x:c r="B28" s="140" t="n">
-        <x:v>46325</x:v>
+        <x:v>46351</x:v>
       </x:c>
       <x:c r="C28" s="137" t="str">
-        <x:v>All website journeys implemented and ready for hardening</x:v>
+        <x:v>Production UI journeys implemented from reusable components and ready for hardening</x:v>
       </x:c>
       <x:c r="D28" s="137" t="str">
-        <x:v>Parallel content, design, and engineering</x:v>
+        <x:v>Controlled overlap across content, design, and engineering</x:v>
       </x:c>
       <x:c r="E28" s="120"/>
       <x:c r="F28" s="120"/>
@@ -1815,7 +1846,7 @@
         <x:v>Core concierge and visual preview</x:v>
       </x:c>
       <x:c r="B29" s="140" t="n">
-        <x:v>46356</x:v>
+        <x:v>46373</x:v>
       </x:c>
       <x:c r="C29" s="137" t="str">
         <x:v>Grounded question answering connected to deterministic preview components</x:v>
@@ -1835,7 +1866,7 @@
         <x:v>All planned features complete</x:v>
       </x:c>
       <x:c r="B30" s="140" t="n">
-        <x:v>46371</x:v>
+        <x:v>46381</x:v>
       </x:c>
       <x:c r="C30" s="137" t="str">
         <x:v>Feature acceptance evidence and evaluation results</x:v>
@@ -1976,7 +2007,7 @@
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="141" t="str">
-        <x:v>Accelerated schedule: working days (Monday–Friday) with controlled task overlap. Phase 1 is feature-complete by 30 October 2026, AI features complete by 15 December 2026, and final release is due 30 December with 31 December contingency.</x:v>
+        <x:v>Resumed schedule: working days (Monday–Friday) with controlled overlap. The preserved mockup is the UI reference. Phase 1 is feature-complete by 25 November 2026, planned AI features complete by 25 December 2026, and final release remains due 30 December with 31 December contingency.</x:v>
       </x:c>
       <x:c r="B3" s="120"/>
       <x:c r="C3" s="120"/>
@@ -2186,16 +2217,16 @@
         <x:v>46274</x:v>
       </x:c>
       <x:c r="I9" s="150" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>On Hold</x:v>
       </x:c>
       <x:c r="J9" s="151" t="str">
-        <x:v>Owner-provided project assets</x:v>
+        <x:v>Owner confirmation, publication rights, and final project materials</x:v>
       </x:c>
       <x:c r="K9" s="151" t="str">
-        <x:v>Confirm copyright, RERA data, pricing policy, and publication permissions.</x:v>
+        <x:v>Confirm copyright, RERA data, pricing policy, publication permission, and final contact details.</x:v>
       </x:c>
       <x:c r="L9" s="151" t="str">
-        <x:v>In progress: building the approved-content register; next evidence is the asset inventory with ownership and publication status.</x:v>
+        <x:v>On hold: the official brochure and existing references are retained, but owner-approved publication content is unavailable. Resume when permission and final materials are received.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
@@ -2273,7 +2304,7 @@
         <x:v>Completed using the approved product brief, sitemap, temporary reference imagery, and an original generated concept board.</x:v>
       </x:c>
       <x:c r="L11" s="151" t="str">
-        <x:v>Completed: Quiet Tropical Modernism direction defines palette, typography, layout, imagery, motifs, components, motion, responsive behavior, and prototype disclosure.</x:v>
+        <x:v>Completed: Quiet Tropical Modernism direction defines the palette, typography, layout, imagery, motifs, components, motion, responsive behavior, and prototype disclosure. The preserved mockup validates the visual direction.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -2312,7 +2343,7 @@
         <x:v>Completed using the Quiet Tropical Modernism direction, WCAG 2.2 AA target, responsive sitemap, and concierge-preview requirements.</x:v>
       </x:c>
       <x:c r="L12" s="151" t="str">
-        <x:v>Completed: machine-readable foundations, responsive grid, typography hierarchy, component contracts, state matrix, accessibility rules, and engineering usage policy delivered.</x:v>
+        <x:v>Completed: machine-readable foundations, responsive grid, typography hierarchy, component contracts, state matrix, accessibility rules, and engineering policy delivered. The preserved mockup is the production UI reference.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
@@ -2326,32 +2357,31 @@
         <x:v>Model project content</x:v>
       </x:c>
       <x:c r="D13" s="151" t="str">
-        <x:v>Create structured models for villas, amenities, plans, locations, contacts, media, and references.</x:v>
+        <x:v>Create evidence-aware models for villas, amenities, plans, locations, contacts, media, and references aligned with the official brochure and preserved mockup sections.</x:v>
       </x:c>
       <x:c r="E13" s="152" t="str">
         <x:v>AKHIL</x:v>
       </x:c>
       <x:c r="F13" s="153" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G13" s="154" t="n">
-        <x:v>46279</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="H13" s="154" t="n">
-        <x:f>WORKDAY(G13,F13-1)</x:f>
-        <x:v>46282</x:v>
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="I13" s="150" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J13" s="151" t="str">
-        <x:v>T0004 and T0005</x:v>
+        <x:v>T0005, official brochure, and available approved references</x:v>
       </x:c>
       <x:c r="K13" s="151" t="str">
-        <x:v>Choose CMS ownership and content approval workflow.</x:v>
+        <x:v>Phase 1 uses repository-managed JSON content with schema validation and evidence metadata. Every unconfirmed field remains provisional.</x:v>
       </x:c>
       <x:c r="L13" s="151" t="str">
-        <x:v>In progress: define structured, evidence-aware records for villas, amenities, plans, locations, contacts, media, documents, and references.</x:v>
+        <x:v>Completed: delivered a versioned JSON Schema, brochure-backed representative records, approval governance, and repository-managed content workflow. T0004 retains owner-dependent publication approval.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="54" customHeight="1">
@@ -2374,11 +2404,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G14" s="154" t="n">
-        <x:v>46286</x:v>
+        <x:v>46300</x:v>
       </x:c>
       <x:c r="H14" s="154" t="n">
-        <x:f>WORKDAY(G14,F14-1)</x:f>
-        <x:v>46287</x:v>
+        <x:v>46301</x:v>
       </x:c>
       <x:c r="I14" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2401,10 +2430,10 @@
         <x:v>T0010</x:v>
       </x:c>
       <x:c r="C15" s="151" t="str">
-        <x:v>Implement core layout</x:v>
+        <x:v>Productionize shared UI</x:v>
       </x:c>
       <x:c r="D15" s="151" t="str">
-        <x:v>Build responsive navigation, footer, page shell, loading states, error states, and reusable sections.</x:v>
+        <x:v>Translate the preserved mockup patterns into reusable responsive navigation, footer, page shell, states, and production sections without modifying the mockup source.</x:v>
       </x:c>
       <x:c r="E15" s="152" t="str">
         <x:v>AKHIL</x:v>
@@ -2413,11 +2442,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G15" s="154" t="n">
-        <x:v>46288</x:v>
+        <x:v>46302</x:v>
       </x:c>
       <x:c r="H15" s="154" t="n">
-        <x:f>WORKDAY(G15,F15-1)</x:f>
-        <x:v>46293</x:v>
+        <x:v>46307</x:v>
       </x:c>
       <x:c r="I15" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2429,7 +2457,7 @@
         <x:v>Confirm final navigation labels and mobile menu behavior.</x:v>
       </x:c>
       <x:c r="L15" s="151" t="str">
-        <x:v>Planned: provide the shared foundation for all pages.</x:v>
+        <x:v>Planned: establish the reusable production UI foundation while keeping the mockup intact as the visual reference.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">
@@ -2440,10 +2468,10 @@
         <x:v>T0011</x:v>
       </x:c>
       <x:c r="C16" s="151" t="str">
-        <x:v>Build homepage</x:v>
+        <x:v>Productionize homepage</x:v>
       </x:c>
       <x:c r="D16" s="151" t="str">
-        <x:v>Create the cinematic hero, project story, highlights, amenities preview, villas preview, location teaser, and conversion actions.</x:v>
+        <x:v>Rebuild the approved mockup homepage experience with reusable components, optimized media, accessible motion, and production content bindings.</x:v>
       </x:c>
       <x:c r="E16" s="152" t="str">
         <x:v>AKHIL</x:v>
@@ -2452,11 +2480,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G16" s="154" t="n">
-        <x:v>46294</x:v>
+        <x:v>46308</x:v>
       </x:c>
       <x:c r="H16" s="154" t="n">
-        <x:f>WORKDAY(G16,F16-1)</x:f>
-        <x:v>46300</x:v>
+        <x:v>46314</x:v>
       </x:c>
       <x:c r="I16" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2468,7 +2495,7 @@
         <x:v>Approve hero media, headline, and primary call to action.</x:v>
       </x:c>
       <x:c r="L16" s="151" t="str">
-        <x:v>Planned: deliver the primary marketing and discovery experience.</x:v>
+        <x:v>Planned: reproduce the approved mockup experience in the real application with maintainable components and verified responsiveness.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="54" customHeight="1">
@@ -2491,11 +2518,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G17" s="154" t="n">
-        <x:v>46296</x:v>
+        <x:v>46310</x:v>
       </x:c>
       <x:c r="H17" s="154" t="n">
-        <x:f>WORKDAY(G17,F17-1)</x:f>
-        <x:v>46300</x:v>
+        <x:v>46314</x:v>
       </x:c>
       <x:c r="I17" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2530,11 +2556,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G18" s="154" t="n">
-        <x:v>46301</x:v>
+        <x:v>46321</x:v>
       </x:c>
       <x:c r="H18" s="154" t="n">
-        <x:f>WORKDAY(G18,F18-1)</x:f>
-        <x:v>46304</x:v>
+        <x:v>46324</x:v>
       </x:c>
       <x:c r="I18" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2569,11 +2594,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G19" s="154" t="n">
-        <x:v>46303</x:v>
+        <x:v>46323</x:v>
       </x:c>
       <x:c r="H19" s="154" t="n">
-        <x:f>WORKDAY(G19,F19-1)</x:f>
-        <x:v>46309</x:v>
+        <x:v>46329</x:v>
       </x:c>
       <x:c r="I19" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2608,11 +2632,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G20" s="154" t="n">
-        <x:v>46307</x:v>
+        <x:v>46328</x:v>
       </x:c>
       <x:c r="H20" s="154" t="n">
-        <x:f>WORKDAY(G20,F20-1)</x:f>
-        <x:v>46309</x:v>
+        <x:v>46330</x:v>
       </x:c>
       <x:c r="I20" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2647,11 +2670,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G21" s="154" t="n">
-        <x:v>46310</x:v>
+        <x:v>46331</x:v>
       </x:c>
       <x:c r="H21" s="154" t="n">
-        <x:f>WORKDAY(G21,F21-1)</x:f>
-        <x:v>46315</x:v>
+        <x:v>46336</x:v>
       </x:c>
       <x:c r="I21" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2686,11 +2708,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G22" s="154" t="n">
-        <x:v>46310</x:v>
+        <x:v>46331</x:v>
       </x:c>
       <x:c r="H22" s="154" t="n">
-        <x:f>WORKDAY(G22,F22-1)</x:f>
-        <x:v>46315</x:v>
+        <x:v>46336</x:v>
       </x:c>
       <x:c r="I22" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2725,11 +2746,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G23" s="154" t="n">
-        <x:v>46316</x:v>
+        <x:v>46337</x:v>
       </x:c>
       <x:c r="H23" s="154" t="n">
-        <x:f>WORKDAY(G23,F23-1)</x:f>
-        <x:v>46318</x:v>
+        <x:v>46339</x:v>
       </x:c>
       <x:c r="I23" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2764,11 +2784,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G24" s="154" t="n">
-        <x:v>46316</x:v>
+        <x:v>46337</x:v>
       </x:c>
       <x:c r="H24" s="154" t="n">
-        <x:f>WORKDAY(G24,F24-1)</x:f>
-        <x:v>46321</x:v>
+        <x:v>46342</x:v>
       </x:c>
       <x:c r="I24" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2803,11 +2822,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G25" s="154" t="n">
-        <x:v>46321</x:v>
+        <x:v>46342</x:v>
       </x:c>
       <x:c r="H25" s="154" t="n">
-        <x:f>WORKDAY(G25,F25-1)</x:f>
-        <x:v>46322</x:v>
+        <x:v>46343</x:v>
       </x:c>
       <x:c r="I25" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2842,11 +2860,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G26" s="154" t="n">
-        <x:v>46321</x:v>
+        <x:v>46342</x:v>
       </x:c>
       <x:c r="H26" s="154" t="n">
-        <x:f>WORKDAY(G26,F26-1)</x:f>
-        <x:v>46323</x:v>
+        <x:v>46344</x:v>
       </x:c>
       <x:c r="I26" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2881,11 +2898,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G27" s="154" t="n">
-        <x:v>46322</x:v>
+        <x:v>46343</x:v>
       </x:c>
       <x:c r="H27" s="154" t="n">
-        <x:f>WORKDAY(G27,F27-1)</x:f>
-        <x:v>46323</x:v>
+        <x:v>46344</x:v>
       </x:c>
       <x:c r="I27" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2920,11 +2936,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G28" s="154" t="n">
-        <x:v>46323</x:v>
+        <x:v>46345</x:v>
       </x:c>
       <x:c r="H28" s="154" t="n">
-        <x:f>WORKDAY(G28,F28-1)</x:f>
-        <x:v>46324</x:v>
+        <x:v>46346</x:v>
       </x:c>
       <x:c r="I28" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2959,11 +2974,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G29" s="154" t="n">
-        <x:v>46323</x:v>
+        <x:v>46345</x:v>
       </x:c>
       <x:c r="H29" s="154" t="n">
-        <x:f>WORKDAY(G29,F29-1)</x:f>
-        <x:v>46324</x:v>
+        <x:v>46346</x:v>
       </x:c>
       <x:c r="I29" s="150" t="str">
         <x:v>Planned</x:v>
@@ -2989,7 +3003,7 @@
         <x:v>Validate responsive layouts</x:v>
       </x:c>
       <x:c r="D30" s="151" t="str">
-        <x:v>Test all templates across desktop, laptop, tablet, Android, and iPhone breakpoints and orientations.</x:v>
+        <x:v>Test production templates against the approved mockup experience across desktop, laptop, tablet, Android, and iPhone breakpoints and orientations.</x:v>
       </x:c>
       <x:c r="E30" s="152" t="str">
         <x:v>AKHIL</x:v>
@@ -2998,11 +3012,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G30" s="154" t="n">
-        <x:v>46324</x:v>
+        <x:v>46349</x:v>
       </x:c>
       <x:c r="H30" s="154" t="n">
-        <x:f>WORKDAY(G30,F30-1)</x:f>
-        <x:v>46325</x:v>
+        <x:v>46350</x:v>
       </x:c>
       <x:c r="I30" s="150" t="str">
         <x:v>Planned</x:v>
@@ -3037,11 +3050,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G31" s="154" t="n">
-        <x:v>46324</x:v>
+        <x:v>46349</x:v>
       </x:c>
       <x:c r="H31" s="154" t="n">
-        <x:f>WORKDAY(G31,F31-1)</x:f>
-        <x:v>46325</x:v>
+        <x:v>46350</x:v>
       </x:c>
       <x:c r="I31" s="150" t="str">
         <x:v>Planned</x:v>
@@ -3076,11 +3088,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G32" s="154" t="n">
-        <x:v>46325</x:v>
+        <x:v>46351</x:v>
       </x:c>
       <x:c r="H32" s="154" t="n">
-        <x:f>WORKDAY(G32,F32-1)</x:f>
-        <x:v>46325</x:v>
+        <x:v>46351</x:v>
       </x:c>
       <x:c r="I32" s="150" t="str">
         <x:v>Planned</x:v>
@@ -3115,11 +3126,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G33" s="159" t="n">
-        <x:v>46325</x:v>
+        <x:v>46351</x:v>
       </x:c>
       <x:c r="H33" s="159" t="n">
-        <x:f>WORKDAY(G33,F33-1)</x:f>
-        <x:v>46325</x:v>
+        <x:v>46351</x:v>
       </x:c>
       <x:c r="I33" s="155" t="str">
         <x:v>Planned</x:v>
@@ -3158,7 +3168,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3399813d43164bb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6b439161d3b4fdf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3215,7 +3225,7 @@
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
       <x:c r="A3" s="141" t="str">
-        <x:v>Accelerated schedule: working days (Monday–Friday) with controlled task overlap. Phase 1 is feature-complete by 30 October 2026, AI features complete by 15 December 2026, and final release is due 30 December with 31 December contingency.</x:v>
+        <x:v>Resumed schedule: working days (Monday–Friday) with controlled overlap. The preserved mockup is the UI reference. Phase 1 is feature-complete by 25 November 2026, planned AI features complete by 25 December 2026, and final release remains due 30 December with 31 December contingency.</x:v>
       </x:c>
       <x:c r="B3" s="120"/>
       <x:c r="C3" s="120"/>
@@ -3301,11 +3311,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G6" s="149" t="n">
-        <x:v>46321</x:v>
+        <x:v>46342</x:v>
       </x:c>
       <x:c r="H6" s="149" t="n">
-        <x:f>WORKDAY(G6,F6-1)</x:f>
-        <x:v>46323</x:v>
+        <x:v>46344</x:v>
       </x:c>
       <x:c r="I6" s="145" t="str">
         <x:v>Not Started</x:v>
@@ -3340,11 +3349,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G7" s="154" t="n">
-        <x:v>46323</x:v>
+        <x:v>46345</x:v>
       </x:c>
       <x:c r="H7" s="154" t="n">
-        <x:f>WORKDAY(G7,F7-1)</x:f>
-        <x:v>46328</x:v>
+        <x:v>46350</x:v>
       </x:c>
       <x:c r="I7" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3379,11 +3387,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G8" s="154" t="n">
-        <x:v>46328</x:v>
+        <x:v>46349</x:v>
       </x:c>
       <x:c r="H8" s="154" t="n">
-        <x:f>WORKDAY(G8,F8-1)</x:f>
-        <x:v>46331</x:v>
+        <x:v>46352</x:v>
       </x:c>
       <x:c r="I8" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3418,11 +3425,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G9" s="154" t="n">
-        <x:v>46330</x:v>
+        <x:v>46351</x:v>
       </x:c>
       <x:c r="H9" s="154" t="n">
-        <x:f>WORKDAY(G9,F9-1)</x:f>
-        <x:v>46336</x:v>
+        <x:v>46357</x:v>
       </x:c>
       <x:c r="I9" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3457,11 +3463,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G10" s="154" t="n">
-        <x:v>46335</x:v>
+        <x:v>46356</x:v>
       </x:c>
       <x:c r="H10" s="154" t="n">
-        <x:f>WORKDAY(G10,F10-1)</x:f>
-        <x:v>46339</x:v>
+        <x:v>46360</x:v>
       </x:c>
       <x:c r="I10" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3496,11 +3501,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G11" s="154" t="n">
-        <x:v>46338</x:v>
+        <x:v>46359</x:v>
       </x:c>
       <x:c r="H11" s="154" t="n">
-        <x:f>WORKDAY(G11,F11-1)</x:f>
-        <x:v>46343</x:v>
+        <x:v>46364</x:v>
       </x:c>
       <x:c r="I11" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3535,11 +3539,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G12" s="154" t="n">
-        <x:v>46342</x:v>
+        <x:v>46363</x:v>
       </x:c>
       <x:c r="H12" s="154" t="n">
-        <x:f>WORKDAY(G12,F12-1)</x:f>
-        <x:v>46346</x:v>
+        <x:v>46367</x:v>
       </x:c>
       <x:c r="I12" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3574,11 +3577,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G13" s="154" t="n">
-        <x:v>46344</x:v>
+        <x:v>46365</x:v>
       </x:c>
       <x:c r="H13" s="154" t="n">
-        <x:f>WORKDAY(G13,F13-1)</x:f>
-        <x:v>46349</x:v>
+        <x:v>46370</x:v>
       </x:c>
       <x:c r="I13" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3613,11 +3615,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G14" s="154" t="n">
-        <x:v>46349</x:v>
+        <x:v>46370</x:v>
       </x:c>
       <x:c r="H14" s="154" t="n">
-        <x:f>WORKDAY(G14,F14-1)</x:f>
-        <x:v>46352</x:v>
+        <x:v>46373</x:v>
       </x:c>
       <x:c r="I14" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3652,11 +3653,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G15" s="154" t="n">
-        <x:v>46349</x:v>
+        <x:v>46370</x:v>
       </x:c>
       <x:c r="H15" s="154" t="n">
-        <x:f>WORKDAY(G15,F15-1)</x:f>
-        <x:v>46352</x:v>
+        <x:v>46373</x:v>
       </x:c>
       <x:c r="I15" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3682,7 +3682,7 @@
         <x:v>Build concierge chat UI</x:v>
       </x:c>
       <x:c r="D16" s="151" t="str">
-        <x:v>Implement responsive messages, streaming, suggested questions, loading, errors, history, feedback, and accessibility.</x:v>
+        <x:v>Implement the production property-assistant chat experience using the preserved mockup bubble and panel behavior as the interaction reference.</x:v>
       </x:c>
       <x:c r="E16" s="152" t="str">
         <x:v>AKHIL</x:v>
@@ -3691,11 +3691,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G16" s="154" t="n">
-        <x:v>46352</x:v>
+        <x:v>46374</x:v>
       </x:c>
       <x:c r="H16" s="154" t="n">
-        <x:f>WORKDAY(G16,F16-1)</x:f>
-        <x:v>46358</x:v>
+        <x:v>46380</x:v>
       </x:c>
       <x:c r="I16" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3721,7 +3720,7 @@
         <x:v>Build dynamic preview panel</x:v>
       </x:c>
       <x:c r="D17" s="151" t="str">
-        <x:v>Render contextual floor plans, images, maps, comparisons, documents, references, and contacts beside the chat.</x:v>
+        <x:v>Render contextual floor plans, images, maps, comparisons, documents, references, and contacts beside the chat using deterministic production components derived from the mockup concept.</x:v>
       </x:c>
       <x:c r="E17" s="152" t="str">
         <x:v>AKHIL</x:v>
@@ -3730,11 +3729,10 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="G17" s="154" t="n">
-        <x:v>46353</x:v>
+        <x:v>46374</x:v>
       </x:c>
       <x:c r="H17" s="154" t="n">
-        <x:f>WORKDAY(G17,F17-1)</x:f>
-        <x:v>46360</x:v>
+        <x:v>46381</x:v>
       </x:c>
       <x:c r="I17" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3769,11 +3767,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G18" s="154" t="n">
-        <x:v>46357</x:v>
+        <x:v>46377</x:v>
       </x:c>
       <x:c r="H18" s="154" t="n">
-        <x:f>WORKDAY(G18,F18-1)</x:f>
-        <x:v>46363</x:v>
+        <x:v>46381</x:v>
       </x:c>
       <x:c r="I18" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3808,11 +3805,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G19" s="154" t="n">
-        <x:v>46359</x:v>
+        <x:v>46377</x:v>
       </x:c>
       <x:c r="H19" s="154" t="n">
-        <x:f>WORKDAY(G19,F19-1)</x:f>
-        <x:v>46365</x:v>
+        <x:v>46381</x:v>
       </x:c>
       <x:c r="I19" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3847,11 +3843,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G20" s="154" t="n">
-        <x:v>46363</x:v>
+        <x:v>46377</x:v>
       </x:c>
       <x:c r="H20" s="154" t="n">
-        <x:f>WORKDAY(G20,F20-1)</x:f>
-        <x:v>46367</x:v>
+        <x:v>46381</x:v>
       </x:c>
       <x:c r="I20" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3886,11 +3881,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G21" s="154" t="n">
-        <x:v>46364</x:v>
+        <x:v>46378</x:v>
       </x:c>
       <x:c r="H21" s="154" t="n">
-        <x:f>WORKDAY(G21,F21-1)</x:f>
-        <x:v>46367</x:v>
+        <x:v>46381</x:v>
       </x:c>
       <x:c r="I21" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3925,11 +3919,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G22" s="154" t="n">
-        <x:v>46365</x:v>
+        <x:v>46379</x:v>
       </x:c>
       <x:c r="H22" s="154" t="n">
-        <x:f>WORKDAY(G22,F22-1)</x:f>
-        <x:v>46370</x:v>
+        <x:v>46384</x:v>
       </x:c>
       <x:c r="I22" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -3964,11 +3957,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G23" s="154" t="n">
-        <x:v>46366</x:v>
+        <x:v>46380</x:v>
       </x:c>
       <x:c r="H23" s="154" t="n">
-        <x:f>WORKDAY(G23,F23-1)</x:f>
-        <x:v>46370</x:v>
+        <x:v>46384</x:v>
       </x:c>
       <x:c r="I23" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -4003,11 +3995,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G24" s="154" t="n">
-        <x:v>46357</x:v>
+        <x:v>46370</x:v>
       </x:c>
       <x:c r="H24" s="154" t="n">
-        <x:f>WORKDAY(G24,F24-1)</x:f>
-        <x:v>46363</x:v>
+        <x:v>46374</x:v>
       </x:c>
       <x:c r="I24" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -4042,11 +4033,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="G25" s="154" t="n">
-        <x:v>46364</x:v>
+        <x:v>46378</x:v>
       </x:c>
       <x:c r="H25" s="154" t="n">
-        <x:f>WORKDAY(G25,F25-1)</x:f>
-        <x:v>46367</x:v>
+        <x:v>46381</x:v>
       </x:c>
       <x:c r="I25" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -4081,11 +4071,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G26" s="154" t="n">
-        <x:v>46366</x:v>
+        <x:v>46377</x:v>
       </x:c>
       <x:c r="H26" s="154" t="n">
-        <x:f>WORKDAY(G26,F26-1)</x:f>
-        <x:v>46372</x:v>
+        <x:v>46381</x:v>
       </x:c>
       <x:c r="I26" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -4120,11 +4109,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G27" s="154" t="n">
-        <x:v>46370</x:v>
+        <x:v>46380</x:v>
       </x:c>
       <x:c r="H27" s="154" t="n">
-        <x:f>WORKDAY(G27,F27-1)</x:f>
-        <x:v>46374</x:v>
+        <x:v>46386</x:v>
       </x:c>
       <x:c r="I27" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -4159,11 +4147,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="G28" s="154" t="n">
-        <x:v>46370</x:v>
+        <x:v>46384</x:v>
       </x:c>
       <x:c r="H28" s="154" t="n">
-        <x:f>WORKDAY(G28,F28-1)</x:f>
-        <x:v>46372</x:v>
+        <x:v>46386</x:v>
       </x:c>
       <x:c r="I28" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -4198,11 +4185,10 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="G29" s="154" t="n">
-        <x:v>46377</x:v>
+        <x:v>46380</x:v>
       </x:c>
       <x:c r="H29" s="154" t="n">
-        <x:f>WORKDAY(G29,F29-1)</x:f>
-        <x:v>46381</x:v>
+        <x:v>46386</x:v>
       </x:c>
       <x:c r="I29" s="150" t="str">
         <x:v>Not Started</x:v>
@@ -4240,7 +4226,6 @@
         <x:v>46384</x:v>
       </x:c>
       <x:c r="H30" s="159" t="n">
-        <x:f>WORKDAY(G30,F30-1)</x:f>
         <x:v>46386</x:v>
       </x:c>
       <x:c r="I30" s="155" t="str">
@@ -4280,7 +4265,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e1d433ce2d84bb4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc8bcae159ab4783"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5028,6 +5013,29 @@
         <x:v>AKHIL</x:v>
       </x:c>
     </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="174" t="str">
+        <x:v>CR030</x:v>
+      </x:c>
+      <x:c r="B35" s="174" t="str">
+        <x:v>Frontend</x:v>
+      </x:c>
+      <x:c r="C35" s="174" t="str">
+        <x:v>Mockup productionization</x:v>
+      </x:c>
+      <x:c r="D35" s="174" t="str">
+        <x:v>Keep the mockup source unchanged as a visual reference. Rebuild approved patterns as reusable, accessible production components with real content contracts.</x:v>
+      </x:c>
+      <x:c r="E35" s="174" t="str">
+        <x:v>Review diff excludes mockup-demo changes; component evidence matches approved desktop and mobile reference behavior.</x:v>
+      </x:c>
+      <x:c r="F35" s="174" t="str">
+        <x:v>Every UI feature</x:v>
+      </x:c>
+      <x:c r="G35" s="179" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
@@ -5035,7 +5043,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7cd557a843b47e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R043f82ea3f1c4d63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6012,7 +6020,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdcf4644420914c9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8ae761156514e14"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Scaffold production web application
T0009
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re07339e2ea1e49c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R04c64ce6f7fc4cef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R6a02233377cd42d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Re80f076b9fa646b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rbff9d76a2e694552"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R30982225fc98455e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re3d462cc74704b3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R34d6295348624684"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R0e1535b3042a4a28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rf5cbfd75b676445b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R55467ec4d3b84958"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rf655f7797dcf463f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,9 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="202" formatCode="dd mmm yyyy"/>
   </x:numFmts>
   <x:fonts count="23">
     <x:font>
@@ -288,7 +289,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="180">
+  <x:cellXfs count="182">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -734,6 +735,12 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="22" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="19" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -2401,25 +2408,25 @@
         <x:v>AKHIL</x:v>
       </x:c>
       <x:c r="F14" s="153" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G14" s="154" t="n">
-        <x:v>46300</x:v>
-      </x:c>
-      <x:c r="H14" s="154" t="n">
-        <x:v>46301</x:v>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G14" s="180" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="H14" s="180" t="n">
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="I14" s="150" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J14" s="151" t="str">
-        <x:v>T0007 technical direction</x:v>
+        <x:v>T0007, T0008, and verified framework compatibility</x:v>
       </x:c>
       <x:c r="K14" s="151" t="str">
-        <x:v>Confirm deployment platform and package manager.</x:v>
+        <x:v>pnpm 12.8.1 confirmed. The production application runs from the repository root; Vercel remains the planned hosting baseline.</x:v>
       </x:c>
       <x:c r="L14" s="151" t="str">
-        <x:v>Planned: establish a production-ready application baseline.</x:v>
+        <x:v>Completed: delivered the Next.js App Router baseline with TypeScript, Tailwind CSS, validated environment and project content, linting, formatting, unit tests, desktop/mobile E2E tests, and a verified production build.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="54" customHeight="1">
@@ -3168,7 +3175,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6b439161d3b4fdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcef2d660a26b43bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4265,7 +4272,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc8bcae159ab4783"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refcd043a58914bb0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5043,7 +5050,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R043f82ea3f1c4d63"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd171a453cf3d47fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5078,7 +5085,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="121" t="str">
-        <x:v>Recommended production baseline. Versions are the latest stable/LTS values verified on 2 September 2026; re-verify before installation or upgrade.</x:v>
+        <x:v>Recommended production baseline. Package versions are re-verified before installation or upgrade; use the Last verified column to identify the review date for each entry.</x:v>
       </x:c>
       <x:c r="B2" s="120"/>
       <x:c r="C2" s="120"/>
@@ -5188,7 +5195,7 @@
         <x:v>Next.js</x:v>
       </x:c>
       <x:c r="F7" s="169" t="str">
-        <x:v>16.3.3</x:v>
+        <x:v>16.3.8</x:v>
       </x:c>
       <x:c r="G7" s="162" t="str">
         <x:v>App Router, server rendering, optimized routing, metadata, images, and deployment flexibility.</x:v>
@@ -5196,8 +5203,8 @@
       <x:c r="H7" s="162" t="str">
         <x:v>https://nextjs.org/blog</x:v>
       </x:c>
-      <x:c r="I7" s="170" t="n">
-        <x:v>46267</x:v>
+      <x:c r="I7" s="181" t="n">
+        <x:v>46298</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
@@ -5217,7 +5224,7 @@
         <x:v>React</x:v>
       </x:c>
       <x:c r="F8" s="169" t="str">
-        <x:v>19.2.7</x:v>
+        <x:v>19.3.0</x:v>
       </x:c>
       <x:c r="G8" s="162" t="str">
         <x:v>Current React release compatible with the selected Next.js baseline.</x:v>
@@ -5225,8 +5232,8 @@
       <x:c r="H8" s="162" t="str">
         <x:v>https://react.dev/versions</x:v>
       </x:c>
-      <x:c r="I8" s="170" t="n">
-        <x:v>46267</x:v>
+      <x:c r="I8" s="181" t="n">
+        <x:v>46298</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
@@ -5246,16 +5253,16 @@
         <x:v>TypeScript</x:v>
       </x:c>
       <x:c r="F9" s="169" t="str">
-        <x:v>7.0.2</x:v>
+        <x:v>6.0.3</x:v>
       </x:c>
       <x:c r="G9" s="162" t="str">
-        <x:v>Strong contracts across UI, API, database, and AI structured outputs.</x:v>
+        <x:v>Latest stable TypeScript release supported by the current framework lint stack. TypeScript 7 is deferred until typescript-eslint support is available.</x:v>
       </x:c>
       <x:c r="H9" s="162" t="str">
         <x:v>https://www.npmjs.com/package/typescript</x:v>
       </x:c>
-      <x:c r="I9" s="170" t="n">
-        <x:v>46267</x:v>
+      <x:c r="I9" s="181" t="n">
+        <x:v>46298</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -5283,8 +5290,8 @@
       <x:c r="H10" s="162" t="str">
         <x:v>https://www.npmjs.com/package/tailwindcss</x:v>
       </x:c>
-      <x:c r="I10" s="170" t="n">
-        <x:v>46267</x:v>
+      <x:c r="I10" s="181" t="n">
+        <x:v>46298</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
@@ -5391,7 +5398,7 @@
         <x:v>Zod</x:v>
       </x:c>
       <x:c r="F14" s="169" t="str">
-        <x:v>4.5.4</x:v>
+        <x:v>4.6.5</x:v>
       </x:c>
       <x:c r="G14" s="162" t="str">
         <x:v>Validate forms, API boundaries, environment variables, and AI outputs.</x:v>
@@ -5399,8 +5406,8 @@
       <x:c r="H14" s="162" t="str">
         <x:v>https://www.npmjs.com/package/zod</x:v>
       </x:c>
-      <x:c r="I14" s="170" t="n">
-        <x:v>46267</x:v>
+      <x:c r="I14" s="181" t="n">
+        <x:v>46298</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
@@ -5710,7 +5717,7 @@
         <x:v>Vitest</x:v>
       </x:c>
       <x:c r="F25" s="169" t="str">
-        <x:v>4.1.11</x:v>
+        <x:v>5.0.3</x:v>
       </x:c>
       <x:c r="G25" s="162" t="str">
         <x:v>Unit and service-level verification with modern TypeScript support.</x:v>
@@ -5718,8 +5725,8 @@
       <x:c r="H25" s="162" t="str">
         <x:v>https://www.npmjs.com/package/vitest</x:v>
       </x:c>
-      <x:c r="I25" s="170" t="n">
-        <x:v>46267</x:v>
+      <x:c r="I25" s="181" t="n">
+        <x:v>46298</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="48" customHeight="1">
@@ -5739,7 +5746,7 @@
         <x:v>Playwright</x:v>
       </x:c>
       <x:c r="F26" s="169" t="str">
-        <x:v>1.62.1</x:v>
+        <x:v>1.63.0</x:v>
       </x:c>
       <x:c r="G26" s="162" t="str">
         <x:v>Responsive, browser, conversion, and AI journey verification.</x:v>
@@ -5747,8 +5754,8 @@
       <x:c r="H26" s="162" t="str">
         <x:v>https://www.npmjs.com/package/@playwright/test</x:v>
       </x:c>
-      <x:c r="I26" s="170" t="n">
-        <x:v>46267</x:v>
+      <x:c r="I26" s="181" t="n">
+        <x:v>46298</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="48" customHeight="1">
@@ -5768,16 +5775,16 @@
         <x:v>ESLint</x:v>
       </x:c>
       <x:c r="F27" s="169" t="str">
-        <x:v>10.9.1</x:v>
+        <x:v>9.39.5</x:v>
       </x:c>
       <x:c r="G27" s="162" t="str">
-        <x:v>Enforce agreed correctness and maintainability rules in CI.</x:v>
+        <x:v>Latest stable ESLint 9 release compatible with the current Next.js lint plugins. ESLint 10 is deferred until the plugin stack supports it.</x:v>
       </x:c>
       <x:c r="H27" s="162" t="str">
         <x:v>https://www.npmjs.com/package/eslint</x:v>
       </x:c>
-      <x:c r="I27" s="170" t="n">
-        <x:v>46267</x:v>
+      <x:c r="I27" s="181" t="n">
+        <x:v>46298</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="48" customHeight="1">
@@ -5797,7 +5804,7 @@
         <x:v>Prettier</x:v>
       </x:c>
       <x:c r="F28" s="169" t="str">
-        <x:v>3.9.6</x:v>
+        <x:v>3.9.9</x:v>
       </x:c>
       <x:c r="G28" s="162" t="str">
         <x:v>Consistent formatting across supported source and content files.</x:v>
@@ -5805,8 +5812,8 @@
       <x:c r="H28" s="162" t="str">
         <x:v>https://www.npmjs.com/package/prettier</x:v>
       </x:c>
-      <x:c r="I28" s="170" t="n">
-        <x:v>46267</x:v>
+      <x:c r="I28" s="181" t="n">
+        <x:v>46298</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="48" customHeight="1">
@@ -6020,7 +6027,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8ae761156514e14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd04e0d09b7a24ac2"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Productionize shared responsive interface
T0010
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re3d462cc74704b3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R34d6295348624684"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R0e1535b3042a4a28"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rf5cbfd75b676445b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R55467ec4d3b84958"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rf655f7797dcf463f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rad822d21f54f4b53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Raa33c5419ee04006"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R1f24dcd39cae48b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Raa0af0020b774d20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R5af9b78878f54f19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R954db6ba1c2d43ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1499,7 +1499,7 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="B8" s="131" t="n">
-        <x:v>7</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="C8" s="120"/>
       <x:c r="D8" s="132" t="str">
@@ -1529,7 +1529,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B9" s="131" t="n">
-        <x:v>20</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C9" s="120"/>
       <x:c r="D9" s="120"/>
@@ -2446,25 +2446,25 @@
         <x:v>AKHIL</x:v>
       </x:c>
       <x:c r="F15" s="153" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="G15" s="154" t="n">
-        <x:v>46302</x:v>
-      </x:c>
-      <x:c r="H15" s="154" t="n">
-        <x:v>46307</x:v>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G15" s="180" t="n">
+        <x:v>46298</x:v>
+      </x:c>
+      <x:c r="H15" s="180" t="n">
+        <x:v>46298</x:v>
       </x:c>
       <x:c r="I15" s="150" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J15" s="151" t="str">
-        <x:v>T0007 and T0009</x:v>
+        <x:v>T0007, T0009, approved sitemap, and preserved mockup reference</x:v>
       </x:c>
       <x:c r="K15" s="151" t="str">
-        <x:v>Confirm final navigation labels and mobile menu behavior.</x:v>
+        <x:v>Primary labels follow the approved sitemap. Mobile navigation uses a full-screen accessible menu; Schedule a Visit remains the dominant action.</x:v>
       </x:c>
       <x:c r="L15" s="151" t="str">
-        <x:v>Planned: establish the reusable production UI foundation while keeping the mockup intact as the visual reference.</x:v>
+        <x:v>Completed: delivered reusable header, mobile navigation, footer, brand, page shell, section heading, action link, preview disclosure, loading/error/not-found states, and shared shells for planned routes. Verified at desktop and mobile widths with unit, E2E, accessibility-aware lint, type, and production-build checks. The mockup source remains unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">
@@ -3175,7 +3175,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcef2d660a26b43bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc9730700b57499c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4272,7 +4272,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refcd043a58914bb0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R66117152295a4863"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5050,7 +5050,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd171a453cf3d47fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8947fcbc39fb4955"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6027,7 +6027,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd04e0d09b7a24ac2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64b63bdcb54c453d"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Build responsive community page
T0012
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rcbe58c0a5db54a29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R0eacabcf77404f89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R005d3a409eeb4f39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R983ef5e30f6442dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R6883b6d3a1e24e4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rbb501ce0d68946c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd810a66c8cb948a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R04a0b9210b554609"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rc1bfb637bbdf4121"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rf3ddb0d86d60426d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R17aab3b60d054ece"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R3c376c061299413f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1499,7 +1499,7 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="B8" s="131" t="n">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C8" s="120"/>
       <x:c r="D8" s="132" t="str">
@@ -1529,7 +1529,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B9" s="131" t="n">
-        <x:v>17</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C9" s="120"/>
       <x:c r="D9" s="120"/>
@@ -2522,25 +2522,25 @@
         <x:v>AKHIL</x:v>
       </x:c>
       <x:c r="F17" s="153" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G17" s="154" t="n">
-        <x:v>46310</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="H17" s="154" t="n">
-        <x:v>46314</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="I17" s="150" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J17" s="151" t="str">
         <x:v>T0008 and T0010</x:v>
       </x:c>
       <x:c r="K17" s="151" t="str">
-        <x:v>Confirm sustainability and security claims with evidence.</x:v>
+        <x:v>Natural ventilation, daylight, landscape, architect, amenity, and security wording is tied to the official brochure. Sustainability certification and installed security systems are not claimed; publication approval remains pending.</x:v>
       </x:c>
       <x:c r="L17" s="151" t="str">
-        <x:v>Planned: communicate the community value proposition clearly.</x:v>
+        <x:v>Completed: replaced the placeholder with a responsive production Community page covering the vision, architectural principles, landscape, shared life, credited architect, and a qualified security section. Added governed content bindings, route metadata, five unit tests in the full suite, seven desktop/mobile browser checks, production build verification, and visual overflow review. The preserved mockup source remains unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="54" customHeight="1">
@@ -3175,7 +3175,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6610e4696b594c7f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f61dccab64548b5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4272,7 +4272,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd51277e265e4ddc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra67e16bbc9964dd6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5050,7 +5050,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra16bd78d20914b51"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R708bb9e68bff48a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6027,7 +6027,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra70d2310011d456f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6447c08b89f64ca9"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Build searchable villas catalogue
T0013
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rd810a66c8cb948a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R04a0b9210b554609"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rc1bfb637bbdf4121"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rf3ddb0d86d60426d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R17aab3b60d054ece"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R3c376c061299413f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R1466a385ddd24584"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rf36af84823734422"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R0191983066b64001"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R23fb70f77e5048ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R65900ab1cf0f4a5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R82c7d6c35b4d4b24"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1499,7 +1499,7 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="B8" s="131" t="n">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C8" s="120"/>
       <x:c r="D8" s="132" t="str">
@@ -1529,7 +1529,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B9" s="131" t="n">
-        <x:v>16</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C9" s="120"/>
       <x:c r="D9" s="120"/>
@@ -2560,25 +2560,25 @@
         <x:v>AKHIL</x:v>
       </x:c>
       <x:c r="F18" s="153" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G18" s="154" t="n">
-        <x:v>46321</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="H18" s="154" t="n">
-        <x:v>46324</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="I18" s="150" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J18" s="151" t="str">
         <x:v>T0008 and villa data approval</x:v>
       </x:c>
       <x:c r="K18" s="151" t="str">
-        <x:v>Confirm villa types, naming, dimensions, and availability rules.</x:v>
+        <x:v>The governed source currently contains one 2,220 sq ft brochure reference plan. Room counts, named variants, price, and availability remain unconfirmed; the catalogue is structured to accept additional approved records later.</x:v>
       </x:c>
       <x:c r="L18" s="151" t="str">
-        <x:v>Planned: enable fast browsing across approved villa options.</x:v>
+        <x:v>Completed: delivered a responsive, searchable villa catalogue with area filtering, honest unknown states, two-level floor breakdown, brochure imagery, empty-state recovery, detail enquiry, and comparison selection prepared for future approved villa types. Seven unit tests, nine desktop/mobile browser checks, production build, and visual overflow review passed. The preserved mockup source remains unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
@@ -3175,7 +3175,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f61dccab64548b5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R321dd508712a473e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4272,7 +4272,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra67e16bbc9964dd6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f0cd4f66e734d45"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5050,7 +5050,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R708bb9e68bff48a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R670a18c6a19a4e8e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6027,7 +6027,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6447c08b89f64ca9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a8bc30cf11f47ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Build villa detail pages
T0014
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R1466a385ddd24584"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rf36af84823734422"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R0191983066b64001"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R23fb70f77e5048ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R65900ab1cf0f4a5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R82c7d6c35b4d4b24"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R845b79148ea34188"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R63bf4e9611da4643"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Re6e1fb505992429a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R4f471108ca4a4f40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R711bfc00141345de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R761651b9d83a4522"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1499,7 +1499,7 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="B8" s="131" t="n">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C8" s="120"/>
       <x:c r="D8" s="132" t="str">
@@ -1529,7 +1529,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B9" s="131" t="n">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C9" s="120"/>
       <x:c r="D9" s="120"/>
@@ -2598,25 +2598,25 @@
         <x:v>AKHIL</x:v>
       </x:c>
       <x:c r="F19" s="153" t="n">
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G19" s="154" t="n">
-        <x:v>46323</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="H19" s="154" t="n">
-        <x:v>46329</x:v>
+        <x:v>46299</x:v>
       </x:c>
       <x:c r="I19" s="150" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J19" s="151" t="str">
         <x:v>T0013 and approved floor plans</x:v>
       </x:c>
       <x:c r="K19" s="151" t="str">
-        <x:v>Confirm whether dimensions and plans need legal disclaimers.</x:v>
+        <x:v>Floor plans are presented as illustrative brochure references. Identity, scale, dimensions, room labels, legal disclaimers, and publication clearance remain subject to confirmation.</x:v>
       </x:c>
       <x:c r="L19" s="151" t="str">
-        <x:v>Planned: provide a complete decision page for each villa type.</x:v>
+        <x:v>Completed: delivered a statically generated villa detail route linked from the catalogue, with brochure gallery, verified floor-area breakdown, two illustrative floor plans, five material-specification groups, contextual enquiry, and clear unknown/legal disclosures. Seven unit tests, eleven desktop/mobile browser checks, production build, and responsive visual review passed. The preserved mockup source remains unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
@@ -3175,7 +3175,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R321dd508712a473e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e7033199b9f47a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4272,7 +4272,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f0cd4f66e734d45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b1b5d37dd45450a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5050,7 +5050,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R670a18c6a19a4e8e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6519b28df906407f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6027,7 +6027,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a8bc30cf11f47ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78c11e9e0f3144f7"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add brochure and contact actions
T0020
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rdf0583e56287497e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R5828f8de32254a08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R7ae835b72f4e40df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R51131e2af9514c5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Ra5570f5ed64a40d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R4a8eac0338cd4581"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rfd87906512a545bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rc7aa580004ab4a9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R3e61811bd7bf4ac1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rcaed50633a174313"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R01ce48c06c2d4402"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rd88a25a8464e4930"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1529,7 +1529,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B9" s="131" t="n">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C9" s="120"/>
       <x:c r="D9" s="120"/>
@@ -1577,7 +1577,7 @@
         <x:v>Blocked / On hold</x:v>
       </x:c>
       <x:c r="B12" s="135" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C12" s="120"/>
       <x:c r="D12" s="120"/>
@@ -2826,25 +2826,23 @@
         <x:v>AKHIL</x:v>
       </x:c>
       <x:c r="F25" s="153" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G25" s="154" t="n">
-        <x:v>46342</x:v>
-      </x:c>
-      <x:c r="H25" s="154" t="n">
-        <x:v>46343</x:v>
-      </x:c>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G25" s="154" t="d">
+        <x:v>2026-10-08T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H25" s="154"/>
       <x:c r="I25" s="150" t="str">
-        <x:v>Planned</x:v>
+        <x:v>On Hold</x:v>
       </x:c>
       <x:c r="J25" s="151" t="str">
         <x:v>Approved brochure and contact details</x:v>
       </x:c>
       <x:c r="K25" s="151" t="str">
-        <x:v>Confirm the official WhatsApp number and prefilled message.</x:v>
+        <x:v>The official brochure identifies two Kerala mobile numbers but does not confirm either as a WhatsApp account. The owner must approve the WhatsApp number and prefilled message before activation.</x:v>
       </x:c>
       <x:c r="L25" s="151" t="str">
-        <x:v>Planned: make high-intent actions visible and measurable.</x:v>
+        <x:v>On hold: delivered the verified official brochure download, two brochure-listed click-to-call links, a brochure-listed email action, responsive action cards, and non-personal interaction events. The WhatsApp action is configuration-ready and remains disabled until owner confirmation. Nineteen unit tests, twenty-seven desktop/mobile browser checks, a production build, responsive visual review, source-file hash verification, and zero-overflow checks passed. The preserved mockup source remains unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="54" customHeight="1">
@@ -3175,7 +3173,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0870937f33e749a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28a3b40b77324ca3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4272,7 +4270,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04da1ef1dfab408d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d9b19058aab4096"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5050,7 +5048,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f23354b4fdb4f96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c43629af3b64a4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6027,7 +6025,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ff168bdeb8a4267"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc845769d011454f"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add integration and E2E coverage
T0026
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Re02597fc1f984ef2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Re2dd601d20af4416"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Re7e0702e5a6d4a32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R2131322d96da4b09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rd5d9648161bd44e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R2f857eedaa4f40d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0b0750cbd1ab41dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rbe576bebb7864b80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R25e2e6b9c1d94b31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R0a6d701c32514f80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R1e16617556c94c77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R855f73426b86461a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1499,7 +1499,7 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="B8" s="131" t="n">
-        <x:v>23</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C8" s="120"/>
       <x:c r="D8" s="132" t="str">
@@ -1529,7 +1529,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B9" s="131" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C9" s="120"/>
       <x:c r="D9" s="120"/>
@@ -3052,25 +3052,25 @@
         <x:v>AKHIL</x:v>
       </x:c>
       <x:c r="F31" s="153" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="G31" s="154" t="n">
-        <x:v>46349</x:v>
-      </x:c>
-      <x:c r="H31" s="154" t="n">
-        <x:v>46350</x:v>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G31" s="154" t="d">
+        <x:v>2026-10-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H31" s="154" t="d">
+        <x:v>2026-10-10T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I31" s="150" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J31" s="151" t="str">
         <x:v>Stable test environment and T0025</x:v>
       </x:c>
       <x:c r="K31" s="151" t="str">
-        <x:v>Confirm test recipients and non-production integrations.</x:v>
+        <x:v>The current enquiry endpoint intentionally stops at preview-only validation and does not transmit data to an external recipient. External map destinations are link-validated without navigating away from the local test environment. Re-run integration tests against approved production services before release.</x:v>
       </x:c>
       <x:c r="L31" s="151" t="str">
-        <x:v>Planned: produce repeatable automated evidence for critical journeys.</x:v>
+        <x:v>Completed: added desktop and mobile integration coverage for the villa-discovery-to-visit journey, governed brochure delivery and browser download, footer policy navigation, unknown-route recovery, enquiry API validation, origin protection, automated-submission rejection, and valid preview-only acceptance. The complete suite now contains fifty browser checks: forty-nine passed with one intended desktop skip. Twenty-five unit tests, production build, lint, TypeScript, formatting, terminology, and route generation checks passed. Added the framework scroll-behavior marker for warning-free route transitions. The preserved mockup source remains unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="54" customHeight="1">
@@ -3173,7 +3173,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad503d85dd5e4dad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cafc36a12f343df"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4270,7 +4270,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78bf09c692b0401c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ddd85854f834c85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5048,7 +5048,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4d5fd43d46b46df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbf552c0bdde4ad7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6025,7 +6025,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b1a2eedddc44f24"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27e2dcc9102d46f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete release candidate UAT
T0027
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0b0750cbd1ab41dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rbe576bebb7864b80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R25e2e6b9c1d94b31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R0a6d701c32514f80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R1e16617556c94c77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R855f73426b86461a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf1450f55e1854689"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rb50f706f27e04708"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R17cfc74714e140ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R945fd75b4fbe4418"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rf99692afe90a40ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Ra7a2352311df4bb1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1499,7 +1499,7 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="B8" s="131" t="n">
-        <x:v>24</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C8" s="120"/>
       <x:c r="D8" s="132" t="str">
@@ -1529,7 +1529,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B9" s="131" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C9" s="120"/>
       <x:c r="D9" s="120"/>
@@ -3092,23 +3092,23 @@
       <x:c r="F32" s="153" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G32" s="154" t="n">
-        <x:v>46351</x:v>
-      </x:c>
-      <x:c r="H32" s="154" t="n">
-        <x:v>46351</x:v>
+      <x:c r="G32" s="154" t="d">
+        <x:v>2026-10-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H32" s="154" t="d">
+        <x:v>2026-10-10T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I32" s="150" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J32" s="151" t="str">
         <x:v>T0026 and stakeholder review</x:v>
       </x:c>
       <x:c r="K32" s="151" t="str">
-        <x:v>Agree severity definitions and acceptance authority.</x:v>
+        <x:v>No stakeholder defects were supplied for this cycle, so acceptance used the approved product brief, governed content, responsive baseline, and existing release criteria. Final owner review and physical-device validation remain release prerequisites.</x:v>
       </x:c>
       <x:c r="L32" s="151" t="str">
-        <x:v>Planned: close release-blocking findings with verification evidence.</x:v>
+        <x:v>Completed: audited all twelve published routes on desktop and mobile for successful rendering, page headings, metadata, image delivery, console errors, internal destinations, compact-navigation closure, and anchored visit positioning. No application defects requiring correction were found. Added repeatable UAT regression coverage. The complete browser suite now contains fifty-six checks: fifty-four passed with two intentional platform-specific skips. Twenty-five unit tests, formatting, lint, TypeScript, and the seventeen-route production build passed. The preserved mockup source remains unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="54" customHeight="1">
@@ -3173,7 +3173,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cafc36a12f343df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d87a5105dd74a81"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4270,7 +4270,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ddd85854f834c85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6cca09575eb4f30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5048,7 +5048,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbf552c0bdde4ad7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc470501aa85246e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6025,7 +6025,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27e2dcc9102d46f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a273d70390e4417"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Prepare Phase 1 release controls
T0028
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf1450f55e1854689"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rb50f706f27e04708"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R17cfc74714e140ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R945fd75b4fbe4418"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rf99692afe90a40ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Ra7a2352311df4bb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf73a0c3b641c4997"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R8128afc898eb45fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R7b20056c32e94c31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R7eacfdc5cef94796"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R59429fd418e34a8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R3de86f961d8841b7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1529,7 +1529,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B9" s="131" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C9" s="120"/>
       <x:c r="D9" s="120"/>
@@ -1577,7 +1577,7 @@
         <x:v>Blocked / On hold</x:v>
       </x:c>
       <x:c r="B12" s="135" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C12" s="120"/>
       <x:c r="D12" s="120"/>
@@ -3130,23 +3130,21 @@
       <x:c r="F33" s="158" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G33" s="159" t="n">
-        <x:v>46351</x:v>
-      </x:c>
-      <x:c r="H33" s="159" t="n">
-        <x:v>46351</x:v>
-      </x:c>
+      <x:c r="G33" s="159" t="d">
+        <x:v>2026-10-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H33" s="159"/>
       <x:c r="I33" s="155" t="str">
-        <x:v>Planned</x:v>
+        <x:v>On Hold</x:v>
       </x:c>
       <x:c r="J33" s="156" t="str">
         <x:v>T0027 accepted</x:v>
       </x:c>
       <x:c r="K33" s="156" t="str">
-        <x:v>Confirm production domain, hosting account, analytics, and launch approval.</x:v>
+        <x:v>Public launch requires written owner publication approval, an approved production domain and hosting account, verified public contact routes, an approved privacy and retention process, an analytics decision, physical-device acceptance, and an authorized production release. The real application is not linked to the preserved mockup hosting project.</x:v>
       </x:c>
       <x:c r="L33" s="156" t="str">
-        <x:v>Planned: publish a responsive, production-ready MVP and baseline metrics.</x:v>
+        <x:v>On hold after release preparation: added a non-cached health endpoint, automated release-quality workflow, environment guidance, monitoring and rollback procedures, backup and recovery position, launch checklist, and release record template. Fifty-six browser checks passed with two intentional platform-specific skips. Twenty-six unit tests, formatting, lint, TypeScript, terminology policy, and the production build passed. Indexing remains disabled by default and no public production deployment was created.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3173,7 +3171,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d87a5105dd74a81"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa8c969fed5d460b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4270,7 +4268,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6cca09575eb4f30"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1446bd0afb26446f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5048,7 +5046,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc470501aa85246e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2aaf7c79ea774d8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6025,7 +6023,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a273d70390e4417"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57f6703662ce4c39"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Record the Phase 1 public release
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf73a0c3b641c4997"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R8128afc898eb45fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R7b20056c32e94c31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R7eacfdc5cef94796"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R59429fd418e34a8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R3de86f961d8841b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rae956246cbd04e6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R75b49d61f82041bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R4cdea7cdaadf4708"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Ra80c4cc71e5243c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R3401f28dbf35456f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R0f7b49072e6a46a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1382,7 +1382,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="121" t="str">
-        <x:v>Production plan resumed on 3 October 2026. The preserved Glitz Pride mockup is the approved UI reference; production release remains targeted for 30 December 2026.</x:v>
+        <x:v>Phase 1 MVP publicly released on 10 October 2026 after owner approval. The preserved Glitz Pride mockup remains unchanged; Phase 2 stays outside the active release.</x:v>
       </x:c>
       <x:c r="B2" s="120"/>
       <x:c r="C2" s="120"/>
@@ -1488,10 +1488,10 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="I7" s="128" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J7" s="128" t="str">
-        <x:v>Mockup-to-production UI acceptance, responsive QA, E2E tests, accessibility, performance, and UAT accepted</x:v>
+        <x:v>Released on Vercel after owner approval, production regression, health, indexing, sitemap, and brochure checks passed</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="52" customHeight="1">
@@ -1499,7 +1499,7 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="B8" s="131" t="n">
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C8" s="120"/>
       <x:c r="D8" s="132" t="str">
@@ -1577,7 +1577,7 @@
         <x:v>Blocked / On hold</x:v>
       </x:c>
       <x:c r="B12" s="135" t="n">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C12" s="120"/>
       <x:c r="D12" s="120"/>
@@ -1892,14 +1892,14 @@
       <x:c r="A31" s="137" t="str">
         <x:v>UAT and production release</x:v>
       </x:c>
-      <x:c r="B31" s="140" t="n">
-        <x:v>46386</x:v>
+      <x:c r="B31" s="140" t="d">
+        <x:v>2026-10-10T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C31" s="137" t="str">
         <x:v>Release checklist, regression results, monitoring, and launch approval</x:v>
       </x:c>
       <x:c r="D31" s="137" t="str">
-        <x:v>Responsive web/PWA; native apps deferred</x:v>
+        <x:v>Public responsive web release completed; Phase 2 remains separately planned</x:v>
       </x:c>
       <x:c r="E31" s="120"/>
       <x:c r="F31" s="120"/>
@@ -3133,18 +3133,20 @@
       <x:c r="G33" s="159" t="d">
         <x:v>2026-10-10T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="H33" s="159"/>
+      <x:c r="H33" s="159" t="d">
+        <x:v>2026-10-10T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="I33" s="155" t="str">
-        <x:v>On Hold</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J33" s="156" t="str">
-        <x:v>T0027 accepted</x:v>
+        <x:v>T0027 accepted. Owner publication approval was relayed by AKHIL on 10 October 2026.</x:v>
       </x:c>
       <x:c r="K33" s="156" t="str">
-        <x:v>Public launch requires written owner publication approval, an approved production domain and hosting account, verified public contact routes, an approved privacy and retention process, an analytics decision, physical-device acceptance, and an authorized production release. The real application is not linked to the preserved mockup hosting project.</x:v>
+        <x:v>Released through the separate glitz-pride-community Vercel project. Analytics and verified WhatsApp routing remain disabled. Existing qualifications and unknown labels remain visible until the owner supplies confirmed details.</x:v>
       </x:c>
       <x:c r="L33" s="156" t="str">
-        <x:v>On hold after release preparation: added a non-cached health endpoint, automated release-quality workflow, environment guidance, monitoring and rollback procedures, backup and recovery position, launch checklist, and release record template. Fifty-six browser checks passed with two intentional platform-specific skips. Twenty-six unit tests, formatting, lint, TypeScript, terminology policy, and the production build passed. Indexing remains disabled by default and no public production deployment was created.</x:v>
+        <x:v>Completed: deployed commit 4721e0b as Vercel deployment dpl_BcQLdbEK6jsGERiiskXCUuMma2W8 and promoted it to https://glitz-pride-community.vercel.app. The public health endpoint, indexing rules, sitemap, canonical metadata, and branded brochure download passed. Fifty-six desktop and mobile browser checks passed with two intentional skips; twenty-six unit tests, formatting, lint, TypeScript, terminology policy, and the production build passed. The preserved mockup source remains unchanged.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -3171,7 +3173,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa8c969fed5d460b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf70eb9d1e4224947"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4268,7 +4270,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1446bd0afb26446f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabba0ead50cf47f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5046,7 +5048,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2aaf7c79ea774d8f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d6d5b57d8ff4cc6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6023,7 +6025,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57f6703662ce4c39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b502fbc0e1d4831"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete the approved content baseline
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rae956246cbd04e6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R75b49d61f82041bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R4cdea7cdaadf4708"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Ra80c4cc71e5243c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R3401f28dbf35456f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R0f7b49072e6a46a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rde2b85c290aa43bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R700f859c29294893"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R58abab62e27b4379"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R9370e42c878449ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R6aaceb6c41f34423"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R9edc6ff526244e04"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1499,7 +1499,7 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="B8" s="131" t="n">
-        <x:v>26</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="C8" s="120"/>
       <x:c r="D8" s="132" t="str">
@@ -1577,7 +1577,7 @@
         <x:v>Blocked / On hold</x:v>
       </x:c>
       <x:c r="B12" s="135" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C12" s="120"/>
       <x:c r="D12" s="120"/>
@@ -2219,21 +2219,20 @@
       <x:c r="G9" s="154" t="n">
         <x:v>46268</x:v>
       </x:c>
-      <x:c r="H9" s="154" t="n">
-        <x:f>WORKDAY(G9,F9-1)</x:f>
-        <x:v>46274</x:v>
+      <x:c r="H9" s="154" t="d">
+        <x:v>2026-10-10T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I9" s="150" t="str">
-        <x:v>On Hold</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J9" s="151" t="str">
-        <x:v>Owner confirmation, publication rights, and final project materials</x:v>
+        <x:v>APR-003 owner approval covers the exact qualified Phase 1 presentation released on 10 October 2026.</x:v>
       </x:c>
       <x:c r="K9" s="151" t="str">
-        <x:v>Confirm copyright, RERA data, pricing policy, publication permission, and final contact details.</x:v>
+        <x:v>Completion approves the current qualified presentation, not every underlying property fact. New media, changed claims, commercial details, contact routes, or removed qualifications require renewed review.</x:v>
       </x:c>
       <x:c r="L9" s="151" t="str">
-        <x:v>On hold: the official brochure and existing references are retained, but owner-approved publication content is unavailable. Resume when permission and final materials are received.</x:v>
+        <x:v>Completed: established the owner-approved Phase 1 content baseline, retained source and qualification labels, preserved unknown pricing, availability, room counts, installed systems, legal status, delivery state, and WhatsApp routing, and updated stale public preview wording. Twenty-six unit tests, formatting, lint, TypeScript, the production build, and fifty-six desktop/mobile browser checks passed with two intentional skips. The preserved mockup source remains unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
@@ -3173,7 +3172,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf70eb9d1e4224947"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a557aaf6dae4e96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4270,7 +4269,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabba0ead50cf47f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra837be311b7a4fa2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5048,7 +5047,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1d6d5b57d8ff4cc6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9cb2e238d124e57"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6025,7 +6024,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b502fbc0e1d4831"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dd0609bda114608"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete Phase 1 contact action tracking
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rde2b85c290aa43bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R700f859c29294893"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R58abab62e27b4379"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R9370e42c878449ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R6aaceb6c41f34423"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R9edc6ff526244e04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R452892db51ec4fce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R57b8c2b246d14e13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rf47de3972a554eb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R930cc151b19849d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rb27ddffbeb794426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rb1b3cf77004e431a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1499,7 +1499,7 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="B8" s="131" t="n">
-        <x:v>27</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="C8" s="120"/>
       <x:c r="D8" s="132" t="str">
@@ -1577,7 +1577,7 @@
         <x:v>Blocked / On hold</x:v>
       </x:c>
       <x:c r="B12" s="135" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C12" s="120"/>
       <x:c r="D12" s="120"/>
@@ -2830,18 +2830,20 @@
       <x:c r="G25" s="154" t="d">
         <x:v>2026-10-08T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="H25" s="154"/>
+      <x:c r="H25" s="180" t="d">
+        <x:v>2026-10-11T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="I25" s="150" t="str">
-        <x:v>On Hold</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J25" s="151" t="str">
-        <x:v>Approved brochure and contact details</x:v>
+        <x:v>Confirmed WhatsApp number +91 98954 68235 supplied by AKHIL on 11 October 2026.</x:v>
       </x:c>
       <x:c r="K25" s="151" t="str">
-        <x:v>The official brochure identifies two Kerala mobile numbers but does not confirm either as a WhatsApp account. The owner must approve the WhatsApp number and prefilled message before activation.</x:v>
+        <x:v>The number is environment-configured with a neutral project-enquiry message. It opens only after a user click and does not include form data. Brochure-listed call and email details remain source-labelled; operating hours and response times are not claimed.</x:v>
       </x:c>
       <x:c r="L25" s="151" t="str">
-        <x:v>On hold: delivered the verified official brochure download, two brochure-listed click-to-call links, a brochure-listed email action, responsive action cards, and non-personal interaction events. The WhatsApp action is configuration-ready and remains disabled until owner confirmation. Nineteen unit tests, twenty-seven desktop/mobile browser checks, a production build, responsive visual review, source-file hash verification, and zero-overflow checks passed. The preserved mockup source remains unchanged.</x:v>
+        <x:v>Completed: enabled and tested the confirmed WhatsApp contact route across desktop and mobile. Unit tests, production build, and 56 browser tests passed; deployment dpl_81JMF65zx2ACiwJ69BH8N3STEkXw was promoted and live health/contact checks passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="54" customHeight="1">
@@ -3172,7 +3174,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a557aaf6dae4e96"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a8d1bd691b4461a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4269,7 +4271,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra837be311b7a4fa2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c102661eae34c50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5047,7 +5049,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9cb2e238d124e57"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b149dfa89d04e45"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6024,7 +6026,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9dd0609bda114608"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0324e5c4ef34ccf"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Define AI concierge use cases
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R452892db51ec4fce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R57b8c2b246d14e13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rf47de3972a554eb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R930cc151b19849d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rb27ddffbeb794426"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rb1b3cf77004e431a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra67b4c386b3b4240"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rbe0dc3e4632244d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R4950b93f7b234e74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R225dbb4e1a954f6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rd0946a19d9b24810"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rb4c6eba844c44280"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -289,7 +289,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="182">
+  <x:cellXfs count="183">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -741,6 +741,9 @@
     </x:xf>
     <x:xf numFmtId="202" fontId="12" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="19" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1382,7 +1385,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="121" t="str">
-        <x:v>Phase 1 MVP publicly released on 10 October 2026 after owner approval. The preserved Glitz Pride mockup remains unchanged; Phase 2 stays outside the active release.</x:v>
+        <x:v>Phase 1 MVP was publicly released on 10 October 2026 after owner approval. Phase 2 AI engineering started early on 11 October 2026; the preserved Glitz Pride mockup remains unchanged.</x:v>
       </x:c>
       <x:c r="B2" s="120"/>
       <x:c r="C2" s="120"/>
@@ -1499,7 +1502,7 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="B8" s="131" t="n">
-        <x:v>28</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C8" s="120"/>
       <x:c r="D8" s="132" t="str">
@@ -1508,8 +1511,8 @@
       <x:c r="E8" s="132" t="str">
         <x:v>Grounded AI concierge with dynamic previews, citations, recommendations, and handoff</x:v>
       </x:c>
-      <x:c r="F8" s="133" t="n">
-        <x:v>46342</x:v>
+      <x:c r="F8" s="133" t="d">
+        <x:v>2026-10-11T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="G8" s="133" t="n">
         <x:v>46386</x:v>
@@ -1518,7 +1521,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="I8" s="132" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J8" s="132" t="str">
         <x:v>AI evaluation, privacy/security review, integration tests, pilot, and UAT accepted</x:v>
@@ -1545,7 +1548,7 @@
         <x:v>Not started</x:v>
       </x:c>
       <x:c r="B10" s="131" t="n">
-        <x:v>25</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="C10" s="120"/>
       <x:c r="D10" s="120"/>
@@ -3174,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a8d1bd691b4461a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfba35eaad2144974"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3314,25 +3317,25 @@
         <x:v>AKHIL</x:v>
       </x:c>
       <x:c r="F6" s="148" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="G6" s="149" t="n">
-        <x:v>46342</x:v>
-      </x:c>
-      <x:c r="H6" s="149" t="n">
-        <x:v>46344</x:v>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G6" s="182" t="d">
+        <x:v>2026-10-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H6" s="182" t="d">
+        <x:v>2026-10-11T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I6" s="145" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J6" s="146" t="str">
-        <x:v>Phase 1 MVP accepted</x:v>
+        <x:v>Phase 1 MVP accepted and publicly released. T0029 started early with full product-scope freedom granted by AKHIL on 11 October 2026.</x:v>
       </x:c>
       <x:c r="K6" s="146" t="str">
-        <x:v>Confirm languages, supported user groups, and prohibited advice.</x:v>
+        <x:v>Approved scope: prospective buyers, families, residents using public information, visitors, overseas prospects, sales/support users, and content administrators. English is the reference language; Malayalam is first, followed by Hindi and Arabic after approved translations and evaluation sets.</x:v>
       </x:c>
       <x:c r="L6" s="146" t="str">
-        <x:v>Not started: begins after the Phase 1 experience and content model stabilize.</x:v>
+        <x:v>Completed: defined 96 testable use cases across 16 intent families, six response modes, five risk tiers, 20 deterministic preview types, escalation routing, cross-intent rules, multilingual boundaries, evaluation-set requirements, and measurable release gates. Automated specification tests and the full quality pipeline passed.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -4271,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c102661eae34c50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff290a20a3674cdf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5049,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b149dfa89d04e45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a88481b112441c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6026,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0324e5c4ef34ccf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea6ebedf60bf4014"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Approve AI knowledge sources
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra67b4c386b3b4240"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rbe0dc3e4632244d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R4950b93f7b234e74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R225dbb4e1a954f6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rd0946a19d9b24810"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rb4c6eba844c44280"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4793ad05ab5a454b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Raeef0054fb9a4384"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R466fd256d5ca4104"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R8725db6c8cb34943"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R2de85ba4c09c4ec1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R36e0c6b097f84389"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfba35eaad2144974"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ced2f485fbc4784"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3335,7 +3335,7 @@
         <x:v>Approved scope: prospective buyers, families, residents using public information, visitors, overseas prospects, sales/support users, and content administrators. English is the reference language; Malayalam is first, followed by Hindi and Arabic after approved translations and evaluation sets.</x:v>
       </x:c>
       <x:c r="L6" s="146" t="str">
-        <x:v>Completed: defined 96 testable use cases across 16 intent families, six response modes, five risk tiers, 20 deterministic preview types, escalation routing, cross-intent rules, multilingual boundaries, evaluation-set requirements, and measurable release gates. Automated specification tests and the full quality pipeline passed.</x:v>
+        <x:v>Completed and expanded: defined 96 governed capability families and exactly 500 executable acceptance cases (194 positive and 306 negative) across all response modes and R0-R4 risk tiers. The deterministic catalogue, strict guardrails, compound attack cases, generator, and automated contracts passed the full quality pipeline. Evidence: docs/ai/concierge-use-cases.md; docs/ai/concierge-evaluation-catalogue.json; commit a7cd5bd.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -3357,23 +3357,23 @@
       <x:c r="F7" s="153" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G7" s="154" t="n">
-        <x:v>46345</x:v>
-      </x:c>
-      <x:c r="H7" s="154" t="n">
-        <x:v>46350</x:v>
+      <x:c r="G7" s="154" t="d">
+        <x:v>2026-10-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H7" s="154" t="d">
+        <x:v>2026-10-11T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I7" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J7" s="151" t="str">
-        <x:v>T0029 and source-owner approval</x:v>
+        <x:v>T0029 completed. APR-003 permits the exact qualified public presentation, while each source remains constrained by its own authority and evidence state.</x:v>
       </x:c>
       <x:c r="K7" s="151" t="str">
-        <x:v>Identify authoritative owners and update frequency for every source.</x:v>
+        <x:v>Resolved: every source now has an authority tier, owner, steward, review trigger, allowed uses, prohibited uses, and retrieval decision. Missing live commercial, legal, operational, privacy, translation, and external-service sources remain blocked.</x:v>
       </x:c>
       <x:c r="L7" s="151" t="str">
-        <x:v>Not started: requires approved, current, and publishable project information.</x:v>
+        <x:v>Completed: catalogued 23 knowledge sources. Five records are retrieval-eligible within explicit qualifications; 17 are pending and blocked; the inactive legacy website is superseded and retained only for provenance. Added conflict, expiry, derivative-source, and index-eligibility rules plus a machine-readable schema and six automated governance tests. Full formatting, 38-test, lint, type-check, production-build, and prohibited-term checks passed. Evidence: docs/ai/knowledge-source-register.md; content/data/ai-knowledge-sources.json; content/schema/ai-knowledge-source.schema.json.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff290a20a3674cdf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b9d376966fa4dae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a88481b112441c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4306de023d544bf2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea6ebedf60bf4014"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e2e86e1e5714479"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Design governed AI knowledge schema
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4793ad05ab5a454b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Raeef0054fb9a4384"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R466fd256d5ca4104"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R8725db6c8cb34943"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R2de85ba4c09c4ec1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R36e0c6b097f84389"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R1ee3b93fb15d4283"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rd88f99d000734645"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R78c8730e1c494c9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R26a9fd1971c143db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Re5c383fd565541f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R724d93a160084e48"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ced2f485fbc4784"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f8d6c803a0a4b77"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3395,23 +3395,23 @@
       <x:c r="F8" s="153" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G8" s="154" t="n">
-        <x:v>46349</x:v>
-      </x:c>
-      <x:c r="H8" s="154" t="n">
-        <x:v>46352</x:v>
+      <x:c r="G8" s="154" t="d">
+        <x:v>2026-10-13T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H8" s="154" t="d">
+        <x:v>2026-10-13T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I8" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J8" s="151" t="str">
-        <x:v>T0030</x:v>
+        <x:v>T0030 completed with 23 governed sources and an explicit retrieval-eligibility boundary.</x:v>
       </x:c>
       <x:c r="K8" s="151" t="str">
-        <x:v>Confirm data classification and retention requirements.</x:v>
+        <x:v>Resolved: classifications are public, internal, confidential, and restricted. Personal conversations and enquiries remain outside the knowledge package until an approved privacy and retention policy exists.</x:v>
       </x:c>
       <x:c r="L8" s="151" t="str">
-        <x:v>Not started: schema will support retrieval, citations, previews, and audits.</x:v>
+        <x:v>Completed: defined vendor-neutral document, chunk, entity, atomic claim, citation, permission, language, lifecycle, embedding-state, and audit-event contracts. Added a brochure-backed reference package with hash-bound citations and seven automated tests covering referential integrity, approved-source eligibility, qualifications, temporal review, numeric units, language state, permissions, and activation audit history. The full formatting, 45-test, lint, type-check, production-build, and prohibited-term checks passed. Evidence: docs/ai/knowledge-schema.md; content/schema/ai-knowledge-package.schema.json; content/data/ai-knowledge-package.sample.json.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b9d376966fa4dae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1090aa193034c36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4306de023d544bf2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69a2da839f594977"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e2e86e1e5714479"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc489461065704d8a"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Build governed AI ingestion pipeline
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R1ee3b93fb15d4283"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rd88f99d000734645"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R78c8730e1c494c9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R26a9fd1971c143db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Re5c383fd565541f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R724d93a160084e48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R82e0ac42c5cf4521"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R57d416a058594215"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R1fdb35e3ff434b47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R100d4edefb3045af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R4816b37088ed49b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R3ae8805915044b75"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f8d6c803a0a4b77"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R690fafc84e684bec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3433,23 +3433,23 @@
       <x:c r="F9" s="153" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G9" s="154" t="n">
-        <x:v>46351</x:v>
-      </x:c>
-      <x:c r="H9" s="154" t="n">
-        <x:v>46357</x:v>
+      <x:c r="G9" s="154" t="d">
+        <x:v>2026-10-13T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H9" s="154" t="d">
+        <x:v>2026-10-13T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I9" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J9" s="151" t="str">
-        <x:v>T0031</x:v>
+        <x:v>T0031 completed with governed document, chunk, permission, lifecycle, citation, and audit contracts.</x:v>
       </x:c>
       <x:c r="K9" s="151" t="str">
-        <x:v>Confirm supported formats and rejection workflow for low-quality inputs.</x:v>
+        <x:v>Resolved: the initial pipeline accepts approved local PDF and JSON sources. Pending, superseded, remote, unsupported, missing, unsafe, parse-failed, and low-quality inputs are quarantined for human review.</x:v>
       </x:c>
       <x:c r="L9" s="151" t="str">
-        <x:v>Not started: ingestion must preserve source traceability and version history.</x:v>
+        <x:v>Completed: built a deterministic ingestion pipeline with approval and path gates, page- and section-level parsing, normalization, stable IDs, SHA-256 hashes, version manifest, source qualifications, audit events, and quarantine evidence. The official nine-page brochure and governed JSON produced 19 retrievable chunks from two eligible sources; 21 other register entries were quarantined. Deterministic replay, 51 tests, lint, type-check, production build, and terminology checks passed. Evidence: scripts/ingest_ai_knowledge.py; docs/ai/ingestion-pipeline.md; content/generated/.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1090aa193034c36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recd4e22759664a0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69a2da839f594977"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R761ab57957244077"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc489461065704d8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35f9a924dc3c4370"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Implement governed vector retrieval
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R82e0ac42c5cf4521"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R57d416a058594215"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R1fdb35e3ff434b47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R100d4edefb3045af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R4816b37088ed49b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R3ae8805915044b75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R8b4348bee7ae4ec3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R9ec4e68bcb9847a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Re4e8068ec2274b32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rb315402966c440f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R851499b2c22447f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R90d980a8468842ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R690fafc84e684bec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09e50bbc27e1460b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3471,23 +3471,23 @@
       <x:c r="F10" s="153" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G10" s="154" t="n">
-        <x:v>46356</x:v>
-      </x:c>
-      <x:c r="H10" s="154" t="n">
-        <x:v>46360</x:v>
+      <x:c r="G10" s="154" t="d">
+        <x:v>2026-10-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H10" s="154" t="d">
+        <x:v>2026-10-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I10" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J10" s="151" t="str">
-        <x:v>T0032 and AI provider credentials</x:v>
+        <x:v>T0032 completed with 19 governed chunks from two approved local sources.</x:v>
       </x:c>
       <x:c r="K10" s="151" t="str">
-        <x:v>Select embedding model, vector dimensions, and hosting approach.</x:v>
+        <x:v>Resolved: use a local multilingual MiniLM sentence model with 384 dimensions and a versioned JSON exact-search index for the current small corpus. Keep the embedding provider configurable and migrate to managed vector storage when scale requires it.</x:v>
       </x:c>
       <x:c r="L10" s="151" t="str">
-        <x:v>Not started: retrieval quality will be measured against approved questions.</x:v>
+        <x:v>Completed: implemented governed embedding eligibility, local multilingual vector generation, a 19-record 384-dimensional index, immutable source-package and index hashes, exact cosine ranking, stable tie breaking, source/document/topic/score/top-k filters, qualification and locator returns, dimension guards, and an optional gateway-compatible runtime provider contract. No billing change or external inference was required. All 56 tests, lint, type-check, production build, and terminology checks passed. Evidence: src/lib/vector-retrieval.ts; scripts/build-vector-index.mjs; content/generated/vector-index.json; docs/ai/vector-retrieval.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recd4e22759664a0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4dcd0f5efee4348"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R761ab57957244077"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R733bcac66cd64a3d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R35f9a924dc3c4370"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73057570c1314d43"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Create retrieval evaluation release gate
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R8b4348bee7ae4ec3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R9ec4e68bcb9847a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Re4e8068ec2274b32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rb315402966c440f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R851499b2c22447f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R90d980a8468842ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7fd70ee8a9fd4cdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R8bd20a38736249b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R44ad57988a8f48c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R1839c7d9985f49a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R1c425bc6929c47c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Ree59a0ae538b4454"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09e50bbc27e1460b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9908fbd28364e65"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3487,7 +3487,7 @@
         <x:v>Resolved: use a local multilingual MiniLM sentence model with 384 dimensions and a versioned JSON exact-search index for the current small corpus. Keep the embedding provider configurable and migrate to managed vector storage when scale requires it.</x:v>
       </x:c>
       <x:c r="L10" s="151" t="str">
-        <x:v>Completed: implemented governed embedding eligibility, local multilingual vector generation, a 19-record 384-dimensional index, immutable source-package and index hashes, exact cosine ranking, stable tie breaking, source/document/topic/score/top-k filters, qualification and locator returns, dimension guards, and an optional gateway-compatible runtime provider contract. No billing change or external inference was required. All 56 tests, lint, type-check, production build, and terminology checks passed. Evidence: src/lib/vector-retrieval.ts; scripts/build-vector-index.mjs; content/generated/vector-index.json; docs/ai/vector-retrieval.md.</x:v>
+        <x:v>Completed: implemented governed embedding eligibility, local multilingual vector generation, a 19-record 384-dimensional index, immutable source-package and index hashes, hybrid semantic and bounded lexical ranking, stable tie breaking, source/document/topic/score/top-k filters, qualification and locator returns, dimension guards, and an optional gateway-compatible runtime provider contract. No billing change or external inference was required. All 56 tests, lint, type-check, production build, and terminology checks passed. Evidence: src/lib/vector-retrieval.ts; scripts/build-vector-index.mjs; content/generated/vector-index.json; docs/ai/vector-retrieval.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
@@ -3509,23 +3509,23 @@
       <x:c r="F11" s="153" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G11" s="154" t="n">
-        <x:v>46359</x:v>
-      </x:c>
-      <x:c r="H11" s="154" t="n">
-        <x:v>46364</x:v>
+      <x:c r="G11" s="154" t="d">
+        <x:v>2026-10-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H11" s="154" t="d">
+        <x:v>2026-10-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I11" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J11" s="151" t="str">
-        <x:v>T0033 and approved answer set</x:v>
+        <x:v>T0033 completed with a governed 19-record multilingual vector index.</x:v>
       </x:c>
       <x:c r="K11" s="151" t="str">
-        <x:v>Define pass thresholds and high-risk question categories.</x:v>
+        <x:v>Resolved: release thresholds are Hit@1 70%, Hit@3 90%, mean reciprocal rank 75%, negative rejection 75%, and citation completeness 100%. R3 and R4 failures require human review.</x:v>
       </x:c>
       <x:c r="L11" s="151" t="str">
-        <x:v>Not started: evaluation becomes the release gate for knowledge changes.</x:v>
+        <x:v>Completed: created 26 locked retrieval cases covering positive and negative scenarios across R0-R4, per-case expected evidence, deterministic offline scoring, relevance and ranking metrics, negative safe-failure checks, citation completeness, immutable index binding, and a failing CI exit. The initial baseline exposed four weaknesses; governed metadata context and a bounded lexical boost corrected retrieval without changing evidence. Final results: Hit@1 83.3%, Hit@3 94.4%, mean reciprocal rank 90.3%, negative rejection 100%, citation completeness 100%. All 61 tests, lint, type-check, production build, and terminology checks passed. Evidence: content/evaluation/; scripts/run-retrieval-evaluation.mjs; docs/ai/retrieval-evaluation.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4dcd0f5efee4348"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86d98ece807d41e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R733bcac66cd64a3d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3391f2b73ce24b1b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73057570c1314d43"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reba5ad90086e4625"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Start grounded Gemini assistant service
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7fd70ee8a9fd4cdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R8bd20a38736249b8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R44ad57988a8f48c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R1839c7d9985f49a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R1c425bc6929c47c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Ree59a0ae538b4454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R426ad5c2f2cc4957"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R8d9c8a518d6642ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R7b207cc9ac9641ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R161f3be1f5594e73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R3002a31f1a5f4b4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rc7f48ef9b5294416"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9908fbd28364e65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84caee56993c41ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3547,23 +3547,21 @@
       <x:c r="F12" s="153" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G12" s="154" t="n">
-        <x:v>46363</x:v>
-      </x:c>
-      <x:c r="H12" s="154" t="n">
-        <x:v>46367</x:v>
-      </x:c>
+      <x:c r="G12" s="154" t="d">
+        <x:v>2026-10-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H12" s="154"/>
       <x:c r="I12" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J12" s="151" t="str">
-        <x:v>T0033 and provider API access</x:v>
+        <x:v>T0033 and T0034 completed. Google Gemini free-tier provider selected; a server-only API key and live provider smoke test remain required.</x:v>
       </x:c>
       <x:c r="K12" s="151" t="str">
-        <x:v>Confirm model selection, budget limits, rate limits, and regional constraints.</x:v>
+        <x:v>Resolved: use stable Gemini 3.8 Flash with free-tier limits, no sensitive personal data, a 0.45 evidence threshold, three citations maximum, six recent turns maximum, and 350 output tokens. Confirm the Google AI Studio key before live testing.</x:v>
       </x:c>
       <x:c r="L12" s="151" t="str">
-        <x:v>Not started: service will expose a controlled API to the website.</x:v>
+        <x:v>In progress: implemented provider-independent conversation orchestration, Gemini generation, governed retrieval invocation, structured answer statuses, opaque session IDs, bounded history, privacy screening, deterministic evidence citations, insufficient-evidence handling, and safe retrieval/provider error recovery. All 69 tests, lint, and type-check pass. Live Gemini verification is pending a server-only API key. Evidence: src/lib/assistant-service.ts; src/lib/assistant-service.test.ts; docs/ai/assistant-service.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
@@ -4274,7 +4272,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86d98ece807d41e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81e071ce8f4e44a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5050,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3391f2b73ce24b1b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49031e6296724282"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6027,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reba5ad90086e4625"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9b3ca02e1b643c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete assistant service tracker task
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R426ad5c2f2cc4957"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R8d9c8a518d6642ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R7b207cc9ac9641ea"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R161f3be1f5594e73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R3002a31f1a5f4b4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rc7f48ef9b5294416"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6daa3a2d76314069"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R70602e6a0f934645"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rd5b29bdb8edf40c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R1070376f7bcb410d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rc27fee0657e84a2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R1f91ffef051a4a6b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84caee56993c41ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19c82a96677a48e1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3550,18 +3550,20 @@
       <x:c r="G12" s="154" t="d">
         <x:v>2026-10-14T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="H12" s="154"/>
+      <x:c r="H12" s="154" t="d">
+        <x:v>2026-10-15T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="I12" s="150" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J12" s="151" t="str">
-        <x:v>T0033 and T0034 completed. Google Gemini free-tier provider selected; a server-only API key and live provider smoke test remain required.</x:v>
+        <x:v>T0033 and T0034 completed. Google Gemini free-tier provider configured with a server-only key in the ignored local environment file. Live provider verification passed.</x:v>
       </x:c>
       <x:c r="K12" s="151" t="str">
-        <x:v>Resolved: use stable Gemini 3.8 Flash with free-tier limits, no sensitive personal data, a 0.45 evidence threshold, three citations maximum, six recent turns maximum, and 350 output tokens. Confirm the Google AI Studio key before live testing.</x:v>
+        <x:v>Resolved: use stable Gemini 3.8 Flash with free-tier limits, no sensitive personal data, a 0.45 evidence threshold, three citations maximum, six recent turns maximum, and 350 output tokens. Temporary provider demand errors return a safe retry response.</x:v>
       </x:c>
       <x:c r="L12" s="151" t="str">
-        <x:v>In progress: implemented provider-independent conversation orchestration, Gemini generation, governed retrieval invocation, structured answer statuses, opaque session IDs, bounded history, privacy screening, deterministic evidence citations, insufficient-evidence handling, and safe retrieval/provider error recovery. All 69 tests, lint, and type-check pass. Live Gemini verification is pending a server-only API key. Evidence: src/lib/assistant-service.ts; src/lib/assistant-service.test.ts; docs/ai/assistant-service.md.</x:v>
+        <x:v>Completed: implemented provider-independent conversation orchestration, Gemini generation, governed retrieval invocation, structured answer statuses, opaque session IDs, bounded history, privacy screening, deterministic evidence citations, insufficient-evidence handling, and safe retrieval/provider error recovery. The server-only key is ignored by Git. Live Google provider authentication and text generation passed with Gemini 3.6 Flash while Gemini 3.8 Flash reported temporary high demand. All 69 tests, formatting, lint, type-check, and production build pass. Evidence: src/lib/assistant-service.ts; src/lib/assistant-service.test.ts; docs/ai/assistant-service.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
@@ -4272,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81e071ce8f4e44a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re031892a7251466d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5050,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49031e6296724282"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba2c529c6c5741de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6027,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9b3ca02e1b643c5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a36dac8fb354658"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add assistant prompt and guardrail policy
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R6daa3a2d76314069"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R70602e6a0f934645"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rd5b29bdb8edf40c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R1070376f7bcb410d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rc27fee0657e84a2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R1f91ffef051a4a6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2572f624c4b74120"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R49a77ef0dcaa4fbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rbfdc08fe44e44756"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R4d686340ba334747"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R668d3ae41ad24ac7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rcec199070ac3413c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19c82a96677a48e1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff6372d9e15c4513"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3585,23 +3585,23 @@
       <x:c r="F13" s="153" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G13" s="154" t="n">
-        <x:v>46365</x:v>
-      </x:c>
-      <x:c r="H13" s="154" t="n">
-        <x:v>46370</x:v>
+      <x:c r="G13" s="154" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H13" s="154" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I13" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J13" s="151" t="str">
-        <x:v>T0029, T0030, and T0035</x:v>
+        <x:v>T0029, T0030, and T0035 completed. The 96 capability families, 500 acceptance cases, governed sources, retrieval controls, and assistant service supplied the policy contract.</x:v>
       </x:c>
       <x:c r="K13" s="151" t="str">
-        <x:v>Approve refusal and escalation language with project stakeholders.</x:v>
+        <x:v>Resolved: policy version 2026-10-16.1 covers instruction hierarchy, untrusted evidence, citations, uncertainty, changing commercial and legal facts, privacy, fair housing, professional boundaries, consent, and human handoff. R4 refusal and R3/R4 escalation occur before retrieval or generation.</x:v>
       </x:c>
       <x:c r="L13" s="151" t="str">
-        <x:v>Not started: prompts and policies will be versioned and evaluated.</x:v>
+        <x:v>Completed: added a versioned server-side instruction policy, deterministic risk classification, pre-retrieval refusal for prompt extraction, private records, deceptive claims, and discriminatory housing requests, plus human-confirmation handling for professional decisions and investment guarantees. Every response now exposes policy version, risk tier, reason code, and handoff requirement. Added focused policy and service tests and implementation documentation. All 79 tests, formatting, lint, type-check, production build, secret scan, terminology scan, and retrieval release thresholds pass. Evidence: src/lib/assistant-policy.ts; src/lib/assistant-policy.test.ts; src/lib/assistant-service.ts; docs/ai/prompt-and-guardrail-policy.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re031892a7251466d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R421ef1de16334a3b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba2c529c6c5741de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R445a9de412894b69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a36dac8fb354658"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24261db2484e4e76"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Implement auditable assistant citations
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R2572f624c4b74120"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R49a77ef0dcaa4fbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rbfdc08fe44e44756"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R4d686340ba334747"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R668d3ae41ad24ac7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rcec199070ac3413c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R8e8ce45d50994aba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rea943fde11c5464b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rac1e7dab2c154220"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R3a9e6879041b4ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R2848cbb3dfe24937"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rcb4c3377a2d640fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff6372d9e15c4513"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20676c1ffc884ee4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3623,23 +3623,23 @@
       <x:c r="F14" s="153" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G14" s="154" t="n">
-        <x:v>46370</x:v>
-      </x:c>
-      <x:c r="H14" s="154" t="n">
-        <x:v>46373</x:v>
+      <x:c r="G14" s="154" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H14" s="154" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I14" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J14" s="151" t="str">
-        <x:v>T0034 through T0036</x:v>
+        <x:v>T0034 through T0036 completed. The evaluated retrieval index, assistant service, and guardrail policy supplied governed evidence and safe unsupported-answer handling.</x:v>
       </x:c>
       <x:c r="K14" s="151" t="str">
-        <x:v>Confirm how citations open documents and protect restricted material.</x:v>
+        <x:v>Resolved: citations open only explicit allow-listed public routes. The public brochure may open in the application; structured or restricted evidence remains auditable by title and locator without exposing an internal path.</x:v>
       </x:c>
       <x:c r="L14" s="151" t="str">
-        <x:v>Not started: every factual project answer must be auditable.</x:v>
+        <x:v>Completed: attached immutable evidence, source, and document IDs; source titles; page or section locators; effective, review, and validity dates; mandatory qualifications; safe optional links; and retrieval-score confidence signals to answered responses. No-evidence and empty-generation paths return no citations, confidence none, and required human handoff. Rebuilt the 19-record index and preserved all release thresholds. All 83 tests, formatting, lint, type-check, production build, terminology scan, and secret scan pass. Evidence: src/lib/assistant-service.ts; src/lib/vector-retrieval.ts; scripts/build-vector-index.mjs; docs/ai/cited-answers.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R421ef1de16334a3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf620400386fe44fe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R445a9de412894b69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2dacdebf86a44cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24261db2484e4e76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbffd2abab8c847e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Define safe assistant preview schema
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R8e8ce45d50994aba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rea943fde11c5464b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rac1e7dab2c154220"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R3a9e6879041b4ca1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R2848cbb3dfe24937"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rcb4c3377a2d640fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R58cde2b1821849d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rd80e630efe7b476a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R3bcc0c4a60724a98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rcfcbfd97da344c30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R46f8ab3e376d482e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R7ca1c7068d1e450b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R20676c1ffc884ee4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82ebddfaae2d44ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3661,23 +3661,23 @@
       <x:c r="F15" s="153" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G15" s="154" t="n">
-        <x:v>46370</x:v>
-      </x:c>
-      <x:c r="H15" s="154" t="n">
-        <x:v>46373</x:v>
+      <x:c r="G15" s="154" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H15" s="154" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I15" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J15" s="151" t="str">
-        <x:v>T0008 and T0035</x:v>
+        <x:v>T0008, T0035, and T0037 completed. The production content modules, assistant service, and cited-answer contract supply trusted records and answer-scoped evidence IDs.</x:v>
       </x:c>
       <x:c r="K15" s="151" t="str">
-        <x:v>Confirm which visual components are permitted for each intent.</x:v>
+        <x:v>Resolved: permitted previews are villa summaries, floor-plan galleries, media galleries, landmark maps, villa comparisons, trusted contact actions, and the approved brochure link. The assistant selects IDs only; application code owns content and presentation.</x:v>
       </x:c>
       <x:c r="L15" s="151" t="str">
-        <x:v>Not started: AI will select approved components instead of generating arbitrary UI.</x:v>
+        <x:v>Completed: created a strict discriminated selection schema and trusted resolver for seven preview families. Unknown fields, arbitrary URLs, text, component names, duplicate IDs, unattached evidence, unregistered records, and non-plan media in plan previews fail closed. Trusted modules supply routes, media, map data, comparisons, contact actions, and document details. Added stable landmark IDs, focused tests, and implementation documentation. All 94 tests, formatting, lint, type-check, production build, terminology scan, secret scan, and retrieval release thresholds pass. Evidence: src/lib/assistant-preview.ts; src/lib/assistant-preview.test.ts; docs/ai/preview-response-schema.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf620400386fe44fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8412d8255fde4e90"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb2dacdebf86a44cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd119426aab2c4c84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbffd2abab8c847e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9949c4963c2b4dbb"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Build responsive concierge chat UI
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R58cde2b1821849d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rd80e630efe7b476a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R3bcc0c4a60724a98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rcfcbfd97da344c30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R46f8ab3e376d482e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R7ca1c7068d1e450b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R58e968546682452d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R953d44050e1445ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R0b5f2916c81641a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R42eec5d848e7468d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Re3d4250039a4499e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R4870660c38d84d13"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82ebddfaae2d44ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R432efba434f0437e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3699,23 +3699,23 @@
       <x:c r="F16" s="153" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G16" s="154" t="n">
-        <x:v>46374</x:v>
-      </x:c>
-      <x:c r="H16" s="154" t="n">
-        <x:v>46380</x:v>
+      <x:c r="G16" s="154" t="d">
+        <x:v>2026-10-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H16" s="154" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I16" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J16" s="151" t="str">
-        <x:v>T0035 and Phase 1 design system</x:v>
+        <x:v>T0035 and the Phase 1 design system are complete. The approved assistant service, local retrieval index, and established responsive UI tokens are integrated.</x:v>
       </x:c>
       <x:c r="K16" s="151" t="str">
-        <x:v>Confirm anonymous versus authenticated conversation history.</x:v>
+        <x:v>Resolved: anonymous conversation history is session-only React memory. It is not stored in browser storage or a database, and only the six latest turns are sent as context.</x:v>
       </x:c>
       <x:c r="L16" s="151" t="str">
-        <x:v>Not started: deliver an approachable concierge experience on all breakpoints.</x:v>
+        <x:v>Completed: added the responsive GP launcher, accessible desktop and mobile conversation drawer, suggested questions, grounded answers with expandable approved sources, focus trapping and restoration, safe error recovery, and the production assistant API connection. Added unit and responsive browser coverage. Retrieval evaluation passed all thresholds; 97 tests, formatting, lint, type-check, production build, and 82 responsive checks passed. Evidence: src/components/assistant/concierge-chat.tsx; src/components/assistant/concierge-chat.css; src/app/api/assistant/route.ts; src/lib/assistant-runtime.ts; docs/ai/concierge-chat-ui.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8412d8255fde4e90"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c1ed15931524837"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd119426aab2c4c84"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d1148a386a74dbc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9949c4963c2b4dbb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc178053286f34cbb"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Build dynamic assistant preview panel
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R58e968546682452d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R953d44050e1445ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R0b5f2916c81641a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R42eec5d848e7468d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Re3d4250039a4499e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R4870660c38d84d13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R9aae34c6be594aac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R32dfe9ac8e574314"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Re8bc81f95d704830"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R4e087c220b804be9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Re3bd14030b2c49dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R4d5cfd1c115d4531"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R432efba434f0437e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec649cddbfd34a7d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3737,23 +3737,23 @@
       <x:c r="F17" s="153" t="n">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="G17" s="154" t="n">
-        <x:v>46374</x:v>
-      </x:c>
-      <x:c r="H17" s="154" t="n">
-        <x:v>46381</x:v>
+      <x:c r="G17" s="154" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H17" s="154" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I17" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J17" s="151" t="str">
-        <x:v>T0038 and T0039</x:v>
+        <x:v>Resolved: T0038 and T0039 are complete. The trusted preview registry, evidence-backed assistant API, local retrieval index, and responsive conversation UI are integrated.</x:v>
       </x:c>
       <x:c r="K17" s="151" t="str">
-        <x:v>Confirm mobile bottom-sheet behavior and fallback when media is unavailable.</x:v>
+        <x:v>Resolved: desktop uses a scroll-contained side panel; mobile uses an accessible in-dialog bottom sheet with a return control. Missing media shows a labeled fallback, and preview selection requires approved evidence.</x:v>
       </x:c>
       <x:c r="L17" s="151" t="str">
-        <x:v>Not started: connect structured AI responses to deterministic visual components.</x:v>
+        <x:v>Completed: connected structured assistant responses to deterministic villa, floor-plan, gallery, location, comparison, contact, and document previews. Added safe single-villa comparison fallback, responsive containment, media error states, component tests, and architecture notes. All 111 tests, formatting, lint, type-check, production build, 88 responsive checks, and all retrieval thresholds across 26 cases passed. Evidence: src/lib/assistant-preview.ts; src/app/api/assistant/route.ts; src/components/assistant/dynamic-preview-panel.tsx; src/components/assistant/concierge-chat.tsx; docs/ai/dynamic-preview-panel.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c1ed15931524837"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R370c9b9f22e3443b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d1148a386a74dbc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73201f8716b7439d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc178053286f34cbb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R158b5ee5c0fa4e11"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add explainable villa recommendations
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R9aae34c6be594aac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R32dfe9ac8e574314"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Re8bc81f95d704830"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R4e087c220b804be9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Re3bd14030b2c49dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R4d5cfd1c115d4531"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc9489cab89144296"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R6a9abe3737134ab8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R1b86f752345a46df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R0d9bbb5e12d541fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rfeb05e9b20a1406f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R8c166de4bfbb4a9d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec649cddbfd34a7d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref17b0dd6c1f4a56"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3775,23 +3775,23 @@
       <x:c r="F18" s="153" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G18" s="154" t="n">
-        <x:v>46377</x:v>
-      </x:c>
-      <x:c r="H18" s="154" t="n">
-        <x:v>46381</x:v>
+      <x:c r="G18" s="154" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H18" s="154" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I18" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J18" s="151" t="str">
-        <x:v>T0037, T0038, and approved villa rules</x:v>
+        <x:v>Resolved: T0037, T0038, and T0040 are complete. Approved catalogue records, answer-scoped evidence IDs, deterministic preview resolution, and the responsive visual panel are integrated.</x:v>
       </x:c>
       <x:c r="K18" s="151" t="str">
-        <x:v>Approve recommendation criteria and prohibit unsupported financial suitability claims.</x:v>
+        <x:v>Resolved: recommendations use neutral property criteria only. Price, affordability, loans, investment value, live availability, protected characteristics, medical or safety suitability, and inferred room capacity are prohibited or routed to qualified human confirmation.</x:v>
       </x:c>
       <x:c r="L18" s="151" t="str">
-        <x:v>Not started: recommendations must be explainable and reproducible.</x:v>
+        <x:v>Completed: added deterministic multi-turn preference collection, explainable match/not-match/unknown criteria, focused clarification, single-approved-option disclosure, numeric mismatch handling, and guarded fallbacks for budget, availability, household size, and unmodelled features. Added the recommendation visual component, tests, responsive coverage, and architecture documentation. All 121 tests, formatting, lint, type-check, production build, 88 responsive checks, and all retrieval thresholds across 26 cases passed. Evidence: src/lib/villa-recommendations.ts; src/lib/assistant-preview.ts; src/app/api/assistant/route.ts; src/components/assistant/dynamic-preview-panel.tsx; docs/ai/villa-recommendations.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R370c9b9f22e3443b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb29b5647bcd44a13"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R73201f8716b7439d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69c319b190904fd1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R158b5ee5c0fa4e11"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae95cd963a1e46fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add safe multilingual assistant foundation
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc9489cab89144296"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R6a9abe3737134ab8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R1b86f752345a46df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R0d9bbb5e12d541fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rfeb05e9b20a1406f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R8c166de4bfbb4a9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra3f51ab680d94493"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R69bd1a16014a4301"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R42371c34784b4f52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R6e2b9f49b7524fe9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rc2b9a07d6853447d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R9179c23e8f8041cd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref17b0dd6c1f4a56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4596f8e0a174368"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3813,23 +3813,23 @@
       <x:c r="F19" s="153" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G19" s="154" t="n">
-        <x:v>46377</x:v>
+      <x:c r="G19" s="154" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="H19" s="154" t="n">
         <x:v>46381</x:v>
       </x:c>
       <x:c r="I19" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J19" s="151" t="str">
-        <x:v>T0037 and translated approved content</x:v>
+        <x:v>T0037 is complete. Language-safe request contracts, detection, retrieval isolation, and guarded fallbacks are implemented. KS-022 approved translated content remains pending.</x:v>
       </x:c>
       <x:c r="K19" s="151" t="str">
-        <x:v>Confirm language priority and translation review owners.</x:v>
+        <x:v>Priority confirmed for implementation: English reference, Malayalam first, then Hindi and Arabic. Pending owner action: name a fluent human translation reviewer and approve versioned translations plus cross-language evaluations.</x:v>
       </x:c>
       <x:c r="L19" s="151" t="str">
-        <x:v>Not started: evaluate factual consistency across every supported language.</x:v>
+        <x:v>In progress: added English, Malayalam, Hindi, and Arabic selection; script detection; API and retrieval language contracts; Arabic RTL metadata; and fail-closed handling that prevents retrieval or model use for unapproved translations. English remains the only approved factual language until KS-022 is approved. Focused validation passed with 128 tests and TypeScript checks. Evidence: src/lib/assistant-language.ts; src/lib/assistant-service.ts; src/lib/vector-retrieval.ts; src/components/assistant/concierge-chat.tsx; docs/ai/multilingual-support.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb29b5647bcd44a13"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b999190d33549d2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R69c319b190904fd1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bcfa923cc2e4eff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae95cd963a1e46fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R649c632bffa447d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Approve multilingual assistant languages
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra3f51ab680d94493"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R69bd1a16014a4301"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R42371c34784b4f52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R6e2b9f49b7524fe9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rc2b9a07d6853447d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R9179c23e8f8041cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R3772a36ed5624207"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Re81fc789bc87480d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R7878763882184acb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R1af19786bd114286"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R330c207adaf74de7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R8399a4a1c6d44d63"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4596f8e0a174368"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc175a42e11a4def"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3816,20 +3816,20 @@
       <x:c r="G19" s="154" t="d">
         <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="H19" s="154" t="n">
-        <x:v>46381</x:v>
+      <x:c r="H19" s="154" t="d">
+        <x:v>2026-10-17T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I19" s="150" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J19" s="151" t="str">
-        <x:v>T0037 is complete. Language-safe request contracts, detection, retrieval isolation, and guarded fallbacks are implemented. KS-022 approved translated content remains pending.</x:v>
+        <x:v>Resolved: T0037 is complete and KS-022 is approved with qualifications. English remains canonical evidence; Malayalam, Hindi, and Arabic response controls are approved and governed.</x:v>
       </x:c>
       <x:c r="K19" s="151" t="str">
-        <x:v>Priority confirmed for implementation: English reference, Malayalam first, then Hindi and Arabic. Pending owner action: name a fluent human translation reviewer and approve versioned translations plus cross-language evaluations.</x:v>
+        <x:v>Resolved: AKHIL confirmed as human reviewer and approval owner for Malayalam, Hindi, and Arabic. Future languages must repeat the same governance, review, RTL/accessibility, safety, and evaluation gates.</x:v>
       </x:c>
       <x:c r="L19" s="151" t="str">
-        <x:v>In progress: added English, Malayalam, Hindi, and Arabic selection; script detection; API and retrieval language contracts; Arabic RTL metadata; and fail-closed handling that prevents retrieval or model use for unapproved translations. English remains the only approved factual language until KS-022 is approved. Focused validation passed with 128 tests and TypeScript checks. Evidence: src/lib/assistant-language.ts; src/lib/assistant-service.ts; src/lib/vector-retrieval.ts; src/components/assistant/concierge-chat.tsx; docs/ai/multilingual-support.md.</x:v>
+        <x:v>Completed: approved Malayalam, Hindi, and Arabic; recorded a versioned translation memory; localized fixed safety and recovery messages; preserved English canonical evidence and citations; enabled multilingual retrieval and target-language generation; retained future-language fail-closed handling; and documented reviewer governance. All 132 tests, formatting, lint, type-check, production build, multilingual retrieval thresholds across 32 cases, and responsive verification passed (87 suite passes plus one isolated rerun pass; 2 intentional desktop navigation skips). Evidence: content/data/approved-translations.json; content/data/ai-knowledge-sources.json; src/lib/assistant-language.ts; src/lib/assistant-service.ts; content/evaluation/retrieval-evaluation-report.json; docs/ai/multilingual-support.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b999190d33549d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b9ff220264542da"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bcfa923cc2e4eff"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb23f5fc5cc26479b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R649c632bffa447d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12a567cb161b4ce4"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add Telugu Tamil and Kannada support
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R3772a36ed5624207"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Re81fc789bc87480d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R7878763882184acb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R1af19786bd114286"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R330c207adaf74de7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R8399a4a1c6d44d63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R7b3b076320ca4129"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rfdc5cf10f4964b6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rfa3d9a2284bc497f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R11910100447b4fed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rc372a15aec534f46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R49901eab70d3409c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc175a42e11a4def"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7d1e3ff5568846a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3805,7 +3805,7 @@
         <x:v>Add multilingual support</x:v>
       </x:c>
       <x:c r="D19" s="151" t="str">
-        <x:v>Support approved project conversations and UI in English, Malayalam, Hindi, and Arabic with language-aware retrieval.</x:v>
+        <x:v>Support approved project conversations and UI in English, Malayalam, Hindi, Arabic, Telugu, Tamil, and Kannada with language-aware retrieval.</x:v>
       </x:c>
       <x:c r="E19" s="152" t="str">
         <x:v>AKHIL</x:v>
@@ -3823,13 +3823,13 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="J19" s="151" t="str">
-        <x:v>Resolved: T0037 is complete and KS-022 is approved with qualifications. English remains canonical evidence; Malayalam, Hindi, and Arabic response controls are approved and governed.</x:v>
+        <x:v>Resolved: T0037 is complete and KS-022 is approved with qualifications. English remains canonical evidence; Malayalam, Hindi, Arabic, Telugu, Tamil, and Kannada response controls are approved and governed.</x:v>
       </x:c>
       <x:c r="K19" s="151" t="str">
-        <x:v>Resolved: AKHIL confirmed as human reviewer and approval owner for Malayalam, Hindi, and Arabic. Future languages must repeat the same governance, review, RTL/accessibility, safety, and evaluation gates.</x:v>
+        <x:v>Resolved: AKHIL is the human reviewer and approval owner for all six non-English languages. Future languages must repeat the same governance, review, direction/accessibility, safety, and evaluation gates.</x:v>
       </x:c>
       <x:c r="L19" s="151" t="str">
-        <x:v>Completed: approved Malayalam, Hindi, and Arabic; recorded a versioned translation memory; localized fixed safety and recovery messages; preserved English canonical evidence and citations; enabled multilingual retrieval and target-language generation; retained future-language fail-closed handling; and documented reviewer governance. All 132 tests, formatting, lint, type-check, production build, multilingual retrieval thresholds across 32 cases, and responsive verification passed (87 suite passes plus one isolated rerun pass; 2 intentional desktop navigation skips). Evidence: content/data/approved-translations.json; content/data/ai-knowledge-sources.json; src/lib/assistant-language.ts; src/lib/assistant-service.ts; content/evaluation/retrieval-evaluation-report.json; docs/ai/multilingual-support.md.</x:v>
+        <x:v>Completed and extended on 2026-10-18: approved Telugu, Tamil, and Kannada in addition to Malayalam, Hindi, and Arabic; added localized fixed safety and recovery messages, script/name detection, interface options, reviewer records, retrieval-only translations, and deterministic evaluation cases. English remains canonical evidence and all citations, names, numbers, units, qualifications, and unknowns are preserved. All 133 tests, formatting, lint, type-check, production build, 88 responsive checks, and all retrieval thresholds across 38 cases passed. Evidence: content/data/approved-translations.json; src/lib/assistant-language.ts; content/evaluation/retrieval-evaluation-cases.json; content/evaluation/retrieval-evaluation-report.json; docs/ai/multilingual-support.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b9ff220264542da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R325168ab19b74bc7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb23f5fc5cc26479b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74960f582dea4145"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12a567cb161b4ce4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref342b7d10764bac"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Build contact reference cards
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rb65d41ff53ee4ada"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R50f83f854a384987"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rd4acd41bf2c94299"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R2bfd1d13aef746ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rbffc1dd0ba714fd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R2148acb996524735"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0838e145f0a843fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Ra1b795c101ac4b5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rde968b9b922e4e50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rb3d68762639e411a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R5ef40d882b7b4f80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rec199f76451640a9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11df8e04489b4883"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d240ca514174d18"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3965,23 +3965,23 @@
       <x:c r="F23" s="153" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="G23" s="154" t="n">
-        <x:v>46380</x:v>
-      </x:c>
-      <x:c r="H23" s="154" t="n">
-        <x:v>46384</x:v>
+      <x:c r="G23" s="154" t="d">
+        <x:v>2026-10-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H23" s="154" t="d">
+        <x:v>2026-10-20T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I23" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J23" s="151" t="str">
-        <x:v>T0038 and public contact consent</x:v>
+        <x:v>Resolved: T0038 and the governed contact-source registry are complete. KS-004 and APR-004 approve the WhatsApp destination. KS-018 remains pending, so brochure phone and email records cannot become current professional contact cards.</x:v>
       </x:c>
       <x:c r="K23" s="151" t="str">
-        <x:v>Confirm permission for names, photographs, and direct contact details.</x:v>
+        <x:v>Resolved: the approved card is department-level and publishes no individual name or photograph. Role and WhatsApp are displayed; languages, working hours, and response time remain Not confirmed. The card cites its source, approval record, and review date. Unapproved requested channels are shown as unavailable.</x:v>
       </x:c>
       <x:c r="L23" s="151" t="str">
-        <x:v>Not started: cards will expose only approved professional information.</x:v>
+        <x:v>Completed: added a typed approved-contact directory, consent-gated department card, explicit unknown fields, source provenance, channel-specific fail-closed behavior, responsive card presentation, safe WhatsApp review action, documentation, and automated coverage. Fixed the voice privacy note contrast after the accessibility audit measured 3.94:1. All 171 unit/component tests, formatting, lint, type-check, production build, 102 responsive checks (100 passed and 2 intentional desktop-navigation skips), and 58 end-to-end/accessibility checks (56 passed and 2 intentional skips) passed. Evidence: src/lib/contact-directory.ts; src/lib/assistant-preview.ts; src/components/assistant/dynamic-preview-panel.tsx; docs/ai/contact-reference-cards.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1363ca01d73a4abf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b950c53a09a48f2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4469a6691cff4fcd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ef4c6882dde4f29"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3aaa7d6d58e14d95"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b2f2a89b5924849"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Build knowledge administration workflow
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R0838e145f0a843fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Ra1b795c101ac4b5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rde968b9b922e4e50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rb3d68762639e411a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R5ef40d882b7b4f80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rec199f76451640a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra3c9cea51c994402"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R3fd1f19d3d0c453b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rab466bc82e6d4a8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rb3501e3175b2483a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R68334fedb98a48fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rfc62b0d286e7475a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d240ca514174d18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R375ae920a2aa4a35"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4003,23 +4003,23 @@
       <x:c r="F24" s="153" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G24" s="154" t="n">
-        <x:v>46370</x:v>
-      </x:c>
-      <x:c r="H24" s="154" t="n">
-        <x:v>46374</x:v>
+      <x:c r="G24" s="154" t="d">
+        <x:v>2026-10-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H24" s="154" t="d">
+        <x:v>2026-10-20T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I24" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J24" s="151" t="str">
-        <x:v>T0031, T0032, and authentication</x:v>
+        <x:v>Resolved: T0031 and T0032 supply the governed schema and ingestion pipeline. Administration authentication uses role-specific environment credentials and fails closed. Production administrator authentication and durable private storage remain intentionally outside this local workflow, so no public administration route is exposed.</x:v>
       </x:c>
       <x:c r="K24" s="151" t="str">
-        <x:v>Confirm administrator roles and approval separation.</x:v>
+        <x:v>Resolved: content-editor and content-reviewer are separate roles, and the reviewer identity must differ from the editor identity. Editors validate, stage, and submit. Reviewers approve, activate, rebuild the index, and roll back. Every action records the actor, role, time, reason, source, and immutable version.</x:v>
       </x:c>
       <x:c r="L24" s="151" t="str">
-        <x:v>Not started: maintain current AI knowledge without developer intervention.</x:v>
+        <x:v>Completed: added a credential-gated local administration command with approved-source checks, JSON and PDF validation, a 20 MB limit, credential-field scanning, SHA-256 version integrity, immutable stored versions, independent review, governed activation, re-index requests, pipeline rebuild execution, audit history, and rollback. The public application remains unchanged and no secret is stored. All 176 unit/component tests, formatting, lint, type-check, and production build passed. Evidence: scripts/knowledge-admin.ts; scripts/knowledge-admin.test.ts; content/administration/knowledge-admin.json; docs/ai/knowledge-administration.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b950c53a09a48f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb506c50fa1004476"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ef4c6882dde4f29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1481b7a326954b29"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b2f2a89b5924849"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c0c9f0b4fe4473c"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Harden AI privacy and security
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Ra3c9cea51c994402"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R3fd1f19d3d0c453b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rab466bc82e6d4a8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rb3501e3175b2483a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R68334fedb98a48fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rfc62b0d286e7475a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc0a255d4c618460d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R7ff50290a5f348d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R1bae209b6c7d4b4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rbfe0e9ecb09942fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R6471850ef4f04759"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R8eb8024a792c44db"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R375ae920a2aa4a35"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c2ae997d7dd481a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4041,23 +4041,23 @@
       <x:c r="F25" s="153" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="G25" s="154" t="n">
-        <x:v>46378</x:v>
-      </x:c>
-      <x:c r="H25" s="154" t="n">
-        <x:v>46381</x:v>
+      <x:c r="G25" s="154" t="d">
+        <x:v>2026-10-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H25" s="154" t="d">
+        <x:v>2026-10-20T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I25" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J25" s="151" t="str">
-        <x:v>T0035, T0044, and threat model</x:v>
+        <x:v>Resolved: T0035 and T0044 are complete. The threat model treats visitor input, conversation history, recordings, forms, retrieved content, provider output, and uploads as untrusted. Public endpoints remain anonymous but cannot store, send, book, or administer; administrative actions remain credential-gated and off the public web surface.</x:v>
       </x:c>
       <x:c r="K25" s="151" t="str">
-        <x:v>Confirm jurisdiction, data residency, retention, and incident-response policy.</x:v>
+        <x:v>Resolved with a fail-closed baseline: jurisdiction, controller, data residency, retention, and rights handling are not yet owner-approved, so KS-020 remains pending and persistent personal-data processing stays disabled. The incident runbook covers endpoint isolation, credential rotation, knowledge rollback, re-indexing, verification, and owner or legal escalation.</x:v>
       </x:c>
       <x:c r="L25" s="151" t="str">
-        <x:v>Not started: complete security review before production data is accepted.</x:v>
+        <x:v>Completed: added shared same-origin, content-type, streamed body-size, per-client throttling, pseudonymous request IDs, no-store and security headers, privacy-safe logs, conversation-wide prompt-injection controls, and abuse detection across assistant, transcription, and enquiry endpoints. Fixed the honeypot branch so automated submissions reach dedicated abuse handling. Added environment controls and documented privacy, incident, and production-limit boundaries. All 187 unit and component tests, formatting, lint, type-check, and production build passed. Evidence: src/lib/api-security.ts; src/lib/assistant-policy.ts; src/lib/assistant-service.ts; src/app/api/assistant/route.ts; src/app/api/assistant/transcribe/route.ts; src/app/api/enquiries/route.ts; docs/ai/privacy-security.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb506c50fa1004476"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f5d9ce41bb344e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1481b7a326954b29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8453033c394f4661"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c0c9f0b4fe4473c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7edaab54bc6047c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Build AI evaluation release gate
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc0a255d4c618460d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R7ff50290a5f348d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R1bae209b6c7d4b4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rbfe0e9ecb09942fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R6471850ef4f04759"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R8eb8024a792c44db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4ca902565af442f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R92ac47188d034105"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R60a65fa97ad94b21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R47e91867778640bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rb8dff13221bd4ac9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rd5911c2e04244d94"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c2ae997d7dd481a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaec9dd17af34639"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4079,23 +4079,23 @@
       <x:c r="F26" s="153" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G26" s="154" t="n">
-        <x:v>46377</x:v>
-      </x:c>
-      <x:c r="H26" s="154" t="n">
-        <x:v>46381</x:v>
+      <x:c r="G26" s="154" t="d">
+        <x:v>2026-10-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H26" s="154" t="d">
+        <x:v>2026-10-20T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I26" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J26" s="151" t="str">
-        <x:v>T0034 and implemented AI features</x:v>
+        <x:v>Resolved: T0034 and the implemented assistant capabilities through T0048 are complete. The suite uses the approved 500-case behavioural catalogue, the governed 38-case retrieval benchmark, and a reviewer-approved 22-case executable response dataset. Routine evaluation is deterministic and makes no external model calls.</x:v>
       </x:c>
       <x:c r="K26" s="151" t="str">
-        <x:v>Approve datasets, thresholds, regression policy, and review cadence.</x:v>
+        <x:v>Resolved: AKHIL approved the executable dataset and strict thresholds. Structured output, policy, citation, grounding, preview, multilingual, recovery, call-budget, and latency gates require 100%. Retrieval keeps its measured thresholds. Run the gate after source, retrieval, prompt, policy, language, model, preview, or security changes and before every public release. Any R3 or R4 miss blocks release and requires review.</x:v>
       </x:c>
       <x:c r="L26" s="151" t="str">
-        <x:v>Not started: prevent unmeasured model or knowledge changes from shipping.</x:v>
+        <x:v>Completed: added an offline multi-layer AI release gate covering 500 behavioural contracts, 38 retrieval cases, and 22 executable assistant scenarios across all seven approved languages. It evaluates grounded claims, citations, refusals, policy risk, structured responses, dynamic previews, failure recovery, latency, and estimated token budgets with zero provider calls. The evaluator exposed and fixed risk-classification gaps for inflected property terms and investment-return guarantees. The gate is wired into release automation. All evaluation suites, 192 unit and component tests, formatting, lint, type-check, and production build passed. Evidence: src/lib/assistant-evaluation.ts; content/evaluation/assistant-response-evaluation-cases.json; scripts/run-ai-evaluation.mjs; content/evaluation/ai-evaluation-release-report.json; docs/ai/ai-evaluation-suite.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7f5d9ce41bb344e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b670d6065c64e72"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8453033c394f4661"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2827b72b87442ec"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7edaab54bc6047c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc95bc637e7814f22"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Run AI integration tests
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R4ca902565af442f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R92ac47188d034105"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R60a65fa97ad94b21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R47e91867778640bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rb8dff13221bd4ac9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Rd5911c2e04244d94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R63e5cf5b402b434e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R75d8439c744e4014"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R85bccbc8679f41a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R8675836eb066497c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R053450e9742843c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R0e78331c6e9548fd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3177,7 +3177,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raaec9dd17af34639"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R428b360fd67444e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4117,23 +4117,23 @@
       <x:c r="F27" s="153" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G27" s="154" t="n">
-        <x:v>46380</x:v>
-      </x:c>
-      <x:c r="H27" s="154" t="n">
-        <x:v>46386</x:v>
+      <x:c r="G27" s="154" t="d">
+        <x:v>2026-10-21T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H27" s="154" t="d">
+        <x:v>2026-10-21T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I27" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J27" s="151" t="str">
-        <x:v>T0039 through T0049</x:v>
+        <x:v>Resolved: T0039 through T0049 are complete. Integration evidence uses deterministic non-production browser fixtures with intercepted assistant responses, no live accounts, API keys, personal data, provider calls, or external transmission.</x:v>
       </x:c>
       <x:c r="K27" s="151" t="str">
-        <x:v>Prepare safe test accounts and non-production integrations.</x:v>
+        <x:v>Resolved: safe integration testing runs in desktop and mobile Chromium with browser route interception. Live-provider staging is intentionally outside this task and requires a separately approved environment, controlled credentials, non-production data, and cost limits.</x:v>
       </x:c>
       <x:c r="L27" s="151" t="str">
-        <x:v>Not started: capture repeatable evidence for end-to-end AI behavior.</x:v>
+        <x:v>Completed: added seven end-to-end AI integration journeys executed across desktop and mobile (14 passing tests): multi-turn context, citations and visual details; explainable recommendations; approved contact routing; editable human handoff; multilingual output; safe refusal; and endpoint failure recovery. The tests exposed and fixed a real session handoff defect where development effect replay consumed the reviewed draft before the enquiry form applied it. The dedicated integration gate, 500-case AI evaluation catalogue, 38 retrieval cases, 22 executable response cases, formatting, lint, type-check, 192 unit/component tests, and production build passed. Evidence: tests/e2e/ai-integration.spec.ts; src/components/contact/enquiry-form.tsx; docs/ai/ai-integration-tests.md; package.json.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="54" customHeight="1">
@@ -4274,7 +4274,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b670d6065c64e72"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89cf2be194cb4f40"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5052,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2827b72b87442ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra71d6ec7865240ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6029,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc95bc637e7814f22"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd918e727922240c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add AI pilot and UAT evidence
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R909f84e65abb4368"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Rfb8173669ab24110"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R8ca4e6e656f74cd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rc0587f951ef7413e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rd76de8591bbc4c0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R474ef64b3c1c4a69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R3540b193904348ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R9d5e7b0c390042e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R3f4db89a1ff74e23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R2f7584c0d9414410"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R35cfba4cc4d7455b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R5ba3688f54dd4cef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,10 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="202" formatCode="dd mmm yyyy"/>
+    <x:numFmt numFmtId="203" formatCode="dd-mmm-yyyy"/>
   </x:numFmts>
   <x:fonts count="23">
     <x:font>
@@ -289,7 +290,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="183">
+  <x:cellXfs count="184">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -743,6 +744,9 @@
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="202" fontId="19" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="19" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top"/>
     </x:xf>
   </x:cellXfs>
@@ -3177,7 +3181,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R715ec85b7a034be5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf83d8bebf22b4e4e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4193,23 +4197,23 @@
       <x:c r="F29" s="153" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G29" s="154" t="n">
-        <x:v>46380</x:v>
+      <x:c r="G29" s="183" t="d">
+        <x:v>2026-10-22T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="H29" s="154" t="n">
         <x:v>46386</x:v>
       </x:c>
       <x:c r="I29" s="150" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="J29" s="151" t="str">
-        <x:v>T0049 through T0051</x:v>
+        <x:v>T0049-T0051 complete. AKHIL is the acceptance authority. Pilot uses synthetic non-personal scenarios on a non-production preview.</x:v>
       </x:c>
       <x:c r="K29" s="151" t="str">
-        <x:v>Select pilot users and define acceptance authority.</x:v>
+        <x:v>Free provider quota or availability must recover before the 12/12 live model-backed acceptance run. Production remains Phase 1 until approval.</x:v>
       </x:c>
       <x:c r="L29" s="151" t="str">
-        <x:v>Not started: release only after evaluation and stakeholder acceptance.</x:v>
+        <x:v>Non-production preview reports Phase 2. Full local gate passed with 203 tests. Hosted desktop and mobile UAT passed 19 tests with 1 expected skip. Deterministic guardrails passed; latest live pilot passed 3/12 because 9 provider-backed cases returned the safe service-unavailable state.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="54" customHeight="1">
@@ -4274,7 +4278,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d4a00ec508e4320"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R701937d5aee84837"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5052,7 +5056,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5428309c72194cc6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re33a19b638ce4991"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6029,7 +6033,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0f2434055c3e4d3c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ea489d6b7c84051"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete AI pilot and UAT
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R3540b193904348ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R9d5e7b0c390042e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R3f4db89a1ff74e23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R2f7584c0d9414410"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R35cfba4cc4d7455b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R5ba3688f54dd4cef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R886608d6faa84031"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R8c4a5828f1ab4947"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rdb040485c33b4bd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R79c84893a4704511"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R7d3163607acd4881"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Ree0b163145c24704"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3181,7 +3181,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf83d8bebf22b4e4e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R624645082d6b4afa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4200,20 +4200,20 @@
       <x:c r="G29" s="183" t="d">
         <x:v>2026-10-22T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="H29" s="154" t="n">
-        <x:v>46386</x:v>
+      <x:c r="H29" s="183" t="d">
+        <x:v>2026-10-22T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I29" s="150" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J29" s="151" t="str">
-        <x:v>T0049-T0051 complete. AKHIL is the acceptance authority. Pilot uses synthetic non-personal scenarios on a non-production preview.</x:v>
+        <x:v>Resolved: T0049-T0051 are complete. AKHIL is the acceptance authority. The pilot used synthetic non-personal scenarios on a non-production preview.</x:v>
       </x:c>
       <x:c r="K29" s="151" t="str">
-        <x:v>Free provider quota or availability must recover before the 12/12 live model-backed acceptance run. Production remains Phase 1 until approval.</x:v>
+        <x:v>Resolved: AKHIL accepted the pilot after one complete 12/12 live run. All approved languages, grounded citations, changing-price handling, strict guardrails, and human confirmation behaved as required. Production promotion remains a separate T0053 decision.</x:v>
       </x:c>
       <x:c r="L29" s="151" t="str">
-        <x:v>Non-production preview reports Phase 2. Full local gate passed with 203 tests. Hosted desktop and mobile UAT passed 19 tests with 1 expected skip. Deterministic guardrails passed; latest live pilot passed 3/12 because 9 provider-backed cases returned the safe service-unavailable state.</x:v>
+        <x:v>Completed: the final live AI pilot passed 12/12 scenarios on the first attempt. Hosted desktop and mobile UAT passed 19 tests with 1 expected skip. The full local gate passed 203 tests and a production build. The release evaluation passed 500 behavioural, 38 retrieval, and 22 executable response cases. Evidence: content/evaluation/ai-pilot-uat-report.json; docs/ai/ai-pilot-uat.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="54" customHeight="1">
@@ -4278,7 +4278,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R701937d5aee84837"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4d258cfbb5d418b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5056,7 +5056,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re33a19b638ce4991"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R525b656f99a7480e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6033,7 +6033,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ea489d6b7c84051"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R784f482c422c4dda"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Define Phase 3 readiness baseline
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rc007030a8f954e2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="Ra5a6c9b6dff943bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R5a0836a6a5f14e6b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R08c69f6273fb49b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rbdfa0c25060b40a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="Re316c3c57c8544ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R273578b0ead34caa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R29ec8333793540ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R548105d511134bf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Racdadb2e607f4740"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R081f9d39377a4af6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R35c0fc6b56564d13"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3 MVP" sheetId="7" r:id="Ra0e8672437fe4d1a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -290,7 +291,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="185">
+  <x:cellXfs count="188">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -752,6 +753,13 @@
     <x:xf numFmtId="203" fontId="19" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top"/>
     </x:xf>
+    <x:xf numFmtId="203" fontId="19" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="12" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1169,6 +1177,26 @@
 </x:table>
 </file>
 
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Phase3Tasks" displayName="Phase3Tasks" ref="A5:L29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="12">
+    <x:tableColumn id="1" name="Index Number"/>
+    <x:tableColumn id="2" name="Task ID"/>
+    <x:tableColumn id="3" name="Task Title"/>
+    <x:tableColumn id="4" name="Task Description"/>
+    <x:tableColumn id="5" name="Task Owner"/>
+    <x:tableColumn id="6" name="Number of Days"/>
+    <x:tableColumn id="7" name="Starting Date"/>
+    <x:tableColumn id="8" name="Ending Date"/>
+    <x:tableColumn id="9" name="Status"/>
+    <x:tableColumn id="10" name="Dependencies"/>
+    <x:tableColumn id="11" name="Clarifications"/>
+    <x:tableColumn id="12" name="Outcome/Comments"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Neutral Project Theme">
   <a:themeElements>
@@ -1392,7 +1420,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="121" t="str">
-        <x:v>Phase 1 MVP was publicly released on 10 October 2026 after owner approval. Phase 2 AI engineering started early on 11 October 2026; the preserved Glitz Pride mockup remains unchanged.</x:v>
+        <x:v>Version 1.0.0 is publicly released and preserved. Phase 3 is planned as a secure owner operations platform; implementation remains paused until AKHIL explicitly authorizes it.</x:v>
       </x:c>
       <x:c r="B2" s="120"/>
       <x:c r="C2" s="120"/>
@@ -1479,7 +1507,7 @@
         <x:v>Total tasks</x:v>
       </x:c>
       <x:c r="B7" s="127" t="n">
-        <x:v>53</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C7" s="120"/>
       <x:c r="D7" s="128" t="str">
@@ -1509,29 +1537,29 @@
         <x:v>Completed</x:v>
       </x:c>
       <x:c r="B8" s="131" t="n">
-        <x:v>29</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C8" s="120"/>
       <x:c r="D8" s="132" t="str">
         <x:v>Phase 2</x:v>
       </x:c>
       <x:c r="E8" s="132" t="str">
-        <x:v>Grounded AI concierge with dynamic previews, citations, recommendations, and handoff</x:v>
-      </x:c>
-      <x:c r="F8" s="133" t="d">
+        <x:v>Grounded AI concierge with dynamic previews, citations, multilingual and voice interaction, evaluations, and controlled handoff</x:v>
+      </x:c>
+      <x:c r="F8" s="186" t="d">
         <x:v>2026-10-11T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="G8" s="133" t="n">
-        <x:v>46386</x:v>
+      <x:c r="G8" s="186" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="H8" s="132" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="I8" s="132" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J8" s="132" t="str">
-        <x:v>AI evaluation, privacy/security review, integration tests, pilot, and UAT accepted</x:v>
+        <x:v>Version 1.0.0 released after 205 tests, 500/38/22 AI evaluations, 12/12 live pilot, 19-pass UAT, and 8/8 production smoke checks</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1539,23 +1567,37 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="B9" s="131" t="n">
-        <x:v>0</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C9" s="120"/>
-      <x:c r="D9" s="120"/>
-      <x:c r="E9" s="120"/>
-      <x:c r="F9" s="120"/>
-      <x:c r="G9" s="120"/>
-      <x:c r="H9" s="120"/>
-      <x:c r="I9" s="120"/>
-      <x:c r="J9" s="120"/>
+      <x:c r="D9" s="120" t="str">
+        <x:v>Phase 3</x:v>
+      </x:c>
+      <x:c r="E9" s="120" t="str">
+        <x:v>Secure owner operations platform covering administration, content, inventory, AI knowledge publishing, enquiries, visits, analytics, and resilience</x:v>
+      </x:c>
+      <x:c r="F9" s="187" t="d">
+        <x:v>2026-10-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G9" s="187" t="d">
+        <x:v>2026-12-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H9" s="120" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="I9" s="120" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J9" s="120" t="str">
+        <x:v>Scope and operating policies approved early on 23 October 2026. Implementation remains paused until AKHIL explicitly authorizes T0056 or the next agreed task.</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="130" t="str">
         <x:v>Not started</x:v>
       </x:c>
       <x:c r="B10" s="131" t="n">
-        <x:v>24</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C10" s="120"/>
       <x:c r="D10" s="120"/>
@@ -3184,7 +3226,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R447349b8ec43405e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b8384a7a18b4f8e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4281,7 +4323,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc7566154baa4862"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3acd7cfa8356486c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5059,7 +5101,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26c043f4e7a948eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfec130c011cc4d80"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6036,7 +6078,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re161b69171df4789"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16b0b94415ec432a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6121,4 +6163,1058 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF2E7D32"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="119" t="str">
+        <x:v>PHASE 3 — SECURE OWNER OPERATIONS PLATFORM MVP</x:v>
+      </x:c>
+      <x:c r="B1" s="120"/>
+      <x:c r="C1" s="120"/>
+      <x:c r="D1" s="120"/>
+      <x:c r="E1" s="120"/>
+      <x:c r="F1" s="120"/>
+      <x:c r="G1" s="120"/>
+      <x:c r="H1" s="120"/>
+      <x:c r="I1" s="120"/>
+      <x:c r="J1" s="120"/>
+      <x:c r="K1" s="120"/>
+      <x:c r="L1" s="120"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="121" t="str">
+        <x:v>Add secure administration, governed content and AI operations, villa inventory, enquiries, visit scheduling, analytics, and production controls.</x:v>
+      </x:c>
+      <x:c r="B2" s="120"/>
+      <x:c r="C2" s="120"/>
+      <x:c r="D2" s="120"/>
+      <x:c r="E2" s="120"/>
+      <x:c r="F2" s="120"/>
+      <x:c r="G2" s="120"/>
+      <x:c r="H2" s="120"/>
+      <x:c r="I2" s="120"/>
+      <x:c r="J2" s="120"/>
+      <x:c r="K2" s="120"/>
+      <x:c r="L2" s="120"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="141" t="str">
+        <x:v>Planned sequence: 26 October–17 December 2026. AKHIL remains the sole owner and reviewer. No Phase 3 implementation starts until AKHIL explicitly authorizes the first task.</x:v>
+      </x:c>
+      <x:c r="B3" s="120"/>
+      <x:c r="C3" s="120"/>
+      <x:c r="D3" s="120"/>
+      <x:c r="E3" s="120"/>
+      <x:c r="F3" s="120"/>
+      <x:c r="G3" s="120"/>
+      <x:c r="H3" s="120"/>
+      <x:c r="I3" s="120"/>
+      <x:c r="J3" s="120"/>
+      <x:c r="K3" s="120"/>
+      <x:c r="L3" s="120"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="120"/>
+      <x:c r="B4" s="120"/>
+      <x:c r="C4" s="120"/>
+      <x:c r="D4" s="120"/>
+      <x:c r="E4" s="120"/>
+      <x:c r="F4" s="120"/>
+      <x:c r="G4" s="120"/>
+      <x:c r="H4" s="120"/>
+      <x:c r="I4" s="120"/>
+      <x:c r="J4" s="120"/>
+      <x:c r="K4" s="120"/>
+      <x:c r="L4" s="120"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="142" t="str">
+        <x:v>Index Number</x:v>
+      </x:c>
+      <x:c r="B5" s="143" t="str">
+        <x:v>Task ID</x:v>
+      </x:c>
+      <x:c r="C5" s="143" t="str">
+        <x:v>Task Title</x:v>
+      </x:c>
+      <x:c r="D5" s="143" t="str">
+        <x:v>Task Description</x:v>
+      </x:c>
+      <x:c r="E5" s="143" t="str">
+        <x:v>Task Owner</x:v>
+      </x:c>
+      <x:c r="F5" s="143" t="str">
+        <x:v>Number of Days</x:v>
+      </x:c>
+      <x:c r="G5" s="143" t="str">
+        <x:v>Starting Date</x:v>
+      </x:c>
+      <x:c r="H5" s="143" t="str">
+        <x:v>Ending Date</x:v>
+      </x:c>
+      <x:c r="I5" s="143" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="J5" s="143" t="str">
+        <x:v>Dependencies</x:v>
+      </x:c>
+      <x:c r="K5" s="143" t="str">
+        <x:v>Clarifications</x:v>
+      </x:c>
+      <x:c r="L5" s="144" t="str">
+        <x:v>Outcome/Comments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="145" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B6" s="145" t="str">
+        <x:v>T0054</x:v>
+      </x:c>
+      <x:c r="C6" s="146" t="str">
+        <x:v>Define Phase 3 scope</x:v>
+      </x:c>
+      <x:c r="D6" s="146" t="str">
+        <x:v>Confirm the mandatory business capabilities, non-goals, acceptance criteria, delivery order, and Version 1 compatibility boundary.</x:v>
+      </x:c>
+      <x:c r="E6" s="147" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F6" s="148" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G6" s="185" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H6" s="185" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I6" s="145" t="str">
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="J6" s="146" t="str">
+        <x:v>Resolved: Version 1.0.0 is tagged and preserved. The Phase 3 tracker contains T0054-T0077, and planning work is isolated on feature/define-phase-3-scope.</x:v>
+      </x:c>
+      <x:c r="K6" s="146" t="str">
+        <x:v>Resolved: AKHIL approved the mandatory scope, explicit non-goals, owner-only initial access, compatibility boundary, acceptance matrix, and definition of done. Implementation remains paused until explicit authorization.</x:v>
+      </x:c>
+      <x:c r="L6" s="146" t="str">
+        <x:v>Completed: defined the full Phase 3 objective, primary users, ten mandatory capability groups, Version 1 compatibility requirements, non-goals, acceptance matrix, and release definition of done. Evidence: docs/phase-3/scope-and-acceptance.md; docs/phase-3/readiness-baseline.md.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="150" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="B7" s="150" t="str">
+        <x:v>T0055</x:v>
+      </x:c>
+      <x:c r="C7" s="151" t="str">
+        <x:v>Approve operating policies</x:v>
+      </x:c>
+      <x:c r="D7" s="151" t="str">
+        <x:v>Define privacy, consent, retention, content authority, commercial-data verification, support ownership, and administrative operating rules.</x:v>
+      </x:c>
+      <x:c r="E7" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F7" s="153" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G7" s="183" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H7" s="183" t="d">
+        <x:v>2026-10-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I7" s="150" t="str">
+        <x:v>Completed</x:v>
+      </x:c>
+      <x:c r="J7" s="151" t="str">
+        <x:v>Resolved: T0054 scope and acceptance boundary are approved. Version 1 privacy-safe AI operations and owner authority remain the baseline.</x:v>
+      </x:c>
+      <x:c r="K7" s="151" t="str">
+        <x:v>Resolved: approved data minimization, consent, initial retention, access, content authority, AI knowledge, enquiry, visit, analytics, incident, and policy-change rules. Periods remain configuration values requiring final legal and owner review before real personal-data collection.</x:v>
+      </x:c>
+      <x:c r="L7" s="151" t="str">
+        <x:v>Completed: established the Phase 3 operating and privacy baseline, initial owner-only role model, synthetic-data rule, editable information inventory, admin navigation, service-selection criteria, environment separation, security controls, budget authority, pre-implementation checklist, and release gate. Evidence: docs/phase-3/operating-policies.md; docs/phase-3/readiness-baseline.md.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="150" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B8" s="150" t="str">
+        <x:v>T0056</x:v>
+      </x:c>
+      <x:c r="C8" s="151" t="str">
+        <x:v>Design secure architecture</x:v>
+      </x:c>
+      <x:c r="D8" s="151" t="str">
+        <x:v>Design the administration, API, database, storage, identity, audit, notification, AI publishing, backup, and deployment boundaries with a threat model.</x:v>
+      </x:c>
+      <x:c r="E8" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F8" s="153" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G8" s="183" t="d">
+        <x:v>2026-10-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H8" s="183" t="d">
+        <x:v>2026-10-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I8" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J8" s="151" t="str">
+        <x:v>T0054-T0055 approved.</x:v>
+      </x:c>
+      <x:c r="K8" s="151" t="str">
+        <x:v>Select managed services only after security, cost, portability, and recovery requirements are reviewed.</x:v>
+      </x:c>
+      <x:c r="L8" s="151" t="str">
+        <x:v>Planned: produce the reviewed architecture, trust boundaries, threat model, service choices, and failure strategy.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="150" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B9" s="150" t="str">
+        <x:v>T0057</x:v>
+      </x:c>
+      <x:c r="C9" s="151" t="str">
+        <x:v>Configure database and storage</x:v>
+      </x:c>
+      <x:c r="D9" s="151" t="str">
+        <x:v>Provision isolated development, preview, and production data services with least-privilege credentials and private managed file storage.</x:v>
+      </x:c>
+      <x:c r="E9" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F9" s="153" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G9" s="183" t="d">
+        <x:v>2026-10-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H9" s="183" t="d">
+        <x:v>2026-10-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I9" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J9" s="151" t="str">
+        <x:v>T0056 architecture approved.</x:v>
+      </x:c>
+      <x:c r="K9" s="151" t="str">
+        <x:v>Confirm region, budget, data residency, storage limits, and separation between public assets and protected documents.</x:v>
+      </x:c>
+      <x:c r="L9" s="151" t="str">
+        <x:v>Planned: configure environment-separated database and storage services without exposing administrative credentials to the browser.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="150" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B10" s="150" t="str">
+        <x:v>T0058</x:v>
+      </x:c>
+      <x:c r="C10" s="151" t="str">
+        <x:v>Implement data schema and migrations</x:v>
+      </x:c>
+      <x:c r="D10" s="151" t="str">
+        <x:v>Create versioned schemas and migrations for users, roles, villas, content, media, documents, enquiries, visits, approvals, notifications, and audits.</x:v>
+      </x:c>
+      <x:c r="E10" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F10" s="153" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G10" s="183" t="d">
+        <x:v>2026-11-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H10" s="183" t="d">
+        <x:v>2026-11-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I10" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J10" s="151" t="str">
+        <x:v>T0057 services configured.</x:v>
+      </x:c>
+      <x:c r="K10" s="151" t="str">
+        <x:v>Define stable identifiers, lifecycle states, ownership, timestamps, deletion rules, and migration rollback requirements.</x:v>
+      </x:c>
+      <x:c r="L10" s="151" t="str">
+        <x:v>Planned: deliver reviewed schemas, constraints, seed strategy, migrations, and rollback-tested development data.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="150" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B11" s="150" t="str">
+        <x:v>T0059</x:v>
+      </x:c>
+      <x:c r="C11" s="151" t="str">
+        <x:v>Add authentication and sessions</x:v>
+      </x:c>
+      <x:c r="D11" s="151" t="str">
+        <x:v>Implement secure administrator sign-in, session expiry, logout, recovery, multi-factor readiness, rate limits, and protected routes.</x:v>
+      </x:c>
+      <x:c r="E11" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F11" s="153" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G11" s="183" t="d">
+        <x:v>2026-11-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H11" s="183" t="d">
+        <x:v>2026-11-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I11" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J11" s="151" t="str">
+        <x:v>T0058 identity tables and environment boundaries ready.</x:v>
+      </x:c>
+      <x:c r="K11" s="151" t="str">
+        <x:v>Confirm the approved identity provider, initial owner account, recovery route, and session duration without storing passwords in application code.</x:v>
+      </x:c>
+      <x:c r="L11" s="151" t="str">
+        <x:v>Planned: provide tested authentication and session security for the owner administration area.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="150" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B12" s="150" t="str">
+        <x:v>T0060</x:v>
+      </x:c>
+      <x:c r="C12" s="151" t="str">
+        <x:v>Enforce role permissions</x:v>
+      </x:c>
+      <x:c r="D12" s="151" t="str">
+        <x:v>Implement server-enforced owner, content, sales, AI reviewer, and read-only permissions using least privilege.</x:v>
+      </x:c>
+      <x:c r="E12" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F12" s="153" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G12" s="183" t="d">
+        <x:v>2026-11-05T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H12" s="183" t="d">
+        <x:v>2026-11-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I12" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J12" s="151" t="str">
+        <x:v>T0059 authentication complete.</x:v>
+      </x:c>
+      <x:c r="K12" s="151" t="str">
+        <x:v>AKHIL must approve the permission matrix and retain sole authority to grant or revoke privileged roles.</x:v>
+      </x:c>
+      <x:c r="L12" s="151" t="str">
+        <x:v>Planned: enforce and test role permissions on every administrative page, API route, record, and sensitive action.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="150" t="n">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B13" s="150" t="str">
+        <x:v>T0061</x:v>
+      </x:c>
+      <x:c r="C13" s="151" t="str">
+        <x:v>Build admin dashboard shell</x:v>
+      </x:c>
+      <x:c r="D13" s="151" t="str">
+        <x:v>Create the responsive administration navigation, overview, loading, empty, error, and permission-denied states.</x:v>
+      </x:c>
+      <x:c r="E13" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F13" s="153" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G13" s="183" t="d">
+        <x:v>2026-11-07T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H13" s="183" t="d">
+        <x:v>2026-11-08T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I13" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J13" s="151" t="str">
+        <x:v>T0059-T0060 security foundations complete.</x:v>
+      </x:c>
+      <x:c r="K13" s="151" t="str">
+        <x:v>The administration design should reuse the product design system while remaining clearly distinct from the public website.</x:v>
+      </x:c>
+      <x:c r="L13" s="151" t="str">
+        <x:v>Planned: deliver an accessible desktop and mobile admin shell with role-aware navigation and operational summaries.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="150" t="n">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="B14" s="150" t="str">
+        <x:v>T0062</x:v>
+      </x:c>
+      <x:c r="C14" s="151" t="str">
+        <x:v>Manage villa inventory</x:v>
+      </x:c>
+      <x:c r="D14" s="151" t="str">
+        <x:v>Add validated create, review, update, archive, availability, construction-status, specification, pricing-status, and verification-date workflows for villas.</x:v>
+      </x:c>
+      <x:c r="E14" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F14" s="153" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G14" s="183" t="d">
+        <x:v>2026-11-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H14" s="183" t="d">
+        <x:v>2026-11-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I14" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J14" s="151" t="str">
+        <x:v>T0058 schema, T0060 permissions, and T0061 shell complete.</x:v>
+      </x:c>
+      <x:c r="K14" s="151" t="str">
+        <x:v>Live price and availability require named authority, verification timestamps, history, and confirmation language before publication.</x:v>
+      </x:c>
+      <x:c r="L14" s="151" t="str">
+        <x:v>Planned: enable governed villa inventory management with history, approvals, and safe public presentation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="150" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="B15" s="150" t="str">
+        <x:v>T0063</x:v>
+      </x:c>
+      <x:c r="C15" s="151" t="str">
+        <x:v>Manage website content</x:v>
+      </x:c>
+      <x:c r="D15" s="151" t="str">
+        <x:v>Add draft, review, approval, publication, scheduling, archival, preview, and rollback workflows for public page content.</x:v>
+      </x:c>
+      <x:c r="E15" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F15" s="153" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G15" s="183" t="d">
+        <x:v>2026-11-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H15" s="183" t="d">
+        <x:v>2026-11-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I15" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J15" s="151" t="str">
+        <x:v>T0061 admin shell and T0060 permissions complete.</x:v>
+      </x:c>
+      <x:c r="K15" s="151" t="str">
+        <x:v>Define which sections are editable, which fields are mandatory, and which changes require owner approval.</x:v>
+      </x:c>
+      <x:c r="L15" s="151" t="str">
+        <x:v>Planned: allow approved content changes without source-code edits while preserving version history and rollback.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="150" t="n">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="B16" s="150" t="str">
+        <x:v>T0064</x:v>
+      </x:c>
+      <x:c r="C16" s="151" t="str">
+        <x:v>Manage media and documents</x:v>
+      </x:c>
+      <x:c r="D16" s="151" t="str">
+        <x:v>Add secure upload, validation, metadata, rights status, replacement, expiry, public/private access, and archival workflows for images and documents.</x:v>
+      </x:c>
+      <x:c r="E16" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F16" s="153" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G16" s="183" t="d">
+        <x:v>2026-11-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H16" s="183" t="d">
+        <x:v>2026-11-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I16" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J16" s="151" t="str">
+        <x:v>T0057 storage and T0062 content lifecycle complete.</x:v>
+      </x:c>
+      <x:c r="K16" s="151" t="str">
+        <x:v>Confirm allowed file types, size limits, malware scanning, image rights, brochure authority, and protected-document rules.</x:v>
+      </x:c>
+      <x:c r="L16" s="151" t="str">
+        <x:v>Planned: deliver rights-aware media and document management with safe URLs, metadata, and lifecycle controls.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="150" t="n">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="B17" s="150" t="str">
+        <x:v>T0065</x:v>
+      </x:c>
+      <x:c r="C17" s="151" t="str">
+        <x:v>Govern AI knowledge publishing</x:v>
+      </x:c>
+      <x:c r="D17" s="151" t="str">
+        <x:v>Create review queues for extracted claims, permissions, qualifications, expiry, conflicts, approval, rejection, activation, and retirement of AI sources.</x:v>
+      </x:c>
+      <x:c r="E17" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F17" s="153" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G17" s="183" t="d">
+        <x:v>2026-11-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H17" s="183" t="d">
+        <x:v>2026-11-19T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I17" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J17" s="151" t="str">
+        <x:v>T0063 document management and existing Phase 2 knowledge contracts available.</x:v>
+      </x:c>
+      <x:c r="K17" s="151" t="str">
+        <x:v>Uploaded material must remain quarantined until an authorized AI reviewer approves its evidence and allowed uses.</x:v>
+      </x:c>
+      <x:c r="L17" s="151" t="str">
+        <x:v>Planned: provide a human-controlled AI knowledge centre that prevents unreviewed sources from reaching retrieval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="150" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="B18" s="150" t="str">
+        <x:v>T0066</x:v>
+      </x:c>
+      <x:c r="C18" s="151" t="str">
+        <x:v>Automate ingestion and indexing</x:v>
+      </x:c>
+      <x:c r="D18" s="151" t="str">
+        <x:v>Connect approved publications to deterministic ingestion, validation, version manifests, embeddings, index rebuilds, rollback, and evidence reports.</x:v>
+      </x:c>
+      <x:c r="E18" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F18" s="153" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G18" s="183" t="d">
+        <x:v>2026-11-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H18" s="183" t="d">
+        <x:v>2026-11-21T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I18" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J18" s="151" t="str">
+        <x:v>T0064 approval workflow and existing ingestion/index pipelines ready.</x:v>
+      </x:c>
+      <x:c r="K18" s="151" t="str">
+        <x:v>Rebuilds must be idempotent, environment-specific, auditable, and unable to replace the active index when validation fails.</x:v>
+      </x:c>
+      <x:c r="L18" s="151" t="str">
+        <x:v>Planned: automate safe knowledge refresh with immutable evidence, activation gates, and last-known-good index recovery.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="150" t="n">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="B19" s="150" t="str">
+        <x:v>T0067</x:v>
+      </x:c>
+      <x:c r="C19" s="151" t="str">
+        <x:v>Add AI release approval gate</x:v>
+      </x:c>
+      <x:c r="D19" s="151" t="str">
+        <x:v>Run retrieval, response, multilingual, safety, citation, preview, and live-provider checks before activating a knowledge or model release.</x:v>
+      </x:c>
+      <x:c r="E19" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F19" s="153" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G19" s="183" t="d">
+        <x:v>2026-11-22T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H19" s="183" t="d">
+        <x:v>2026-11-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I19" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J19" s="151" t="str">
+        <x:v>T0065 automated indexing and Phase 2 evaluation suites available.</x:v>
+      </x:c>
+      <x:c r="K19" s="151" t="str">
+        <x:v>AKHIL is the final AI release approver; critical policy, grounding, privacy, or citation failures must block activation.</x:v>
+      </x:c>
+      <x:c r="L19" s="151" t="str">
+        <x:v>Planned: add a reviewer-visible approval gate with comparable results, sign-off, rejection reasons, and rollback.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="150" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="B20" s="150" t="str">
+        <x:v>T0068</x:v>
+      </x:c>
+      <x:c r="C20" s="151" t="str">
+        <x:v>Manage enquiries</x:v>
+      </x:c>
+      <x:c r="D20" s="151" t="str">
+        <x:v>Build consented enquiry capture, assignment, status, notes, follow-up, export, retention, deletion, and controlled contact workflows.</x:v>
+      </x:c>
+      <x:c r="E20" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F20" s="153" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G20" s="183" t="d">
+        <x:v>2026-11-24T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H20" s="183" t="d">
+        <x:v>2026-11-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I20" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J20" s="151" t="str">
+        <x:v>T0055 privacy rules, T0058 schema, T0060 permissions, and T0061 shell complete.</x:v>
+      </x:c>
+      <x:c r="K20" s="151" t="str">
+        <x:v>Collect only necessary contact data; confirm consent text, approved contact channels, retention, deletion, and staff access.</x:v>
+      </x:c>
+      <x:c r="L20" s="151" t="str">
+        <x:v>Planned: provide privacy-governed enquiry management from visitor submission through reviewed closure.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="150" t="n">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="B21" s="150" t="str">
+        <x:v>T0069</x:v>
+      </x:c>
+      <x:c r="C21" s="151" t="str">
+        <x:v>Schedule site visits</x:v>
+      </x:c>
+      <x:c r="D21" s="151" t="str">
+        <x:v>Add owner-controlled availability, slot capacity, request, confirmation, rescheduling, cancellation, reminders, and assigned representative workflows.</x:v>
+      </x:c>
+      <x:c r="E21" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F21" s="153" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G21" s="183" t="d">
+        <x:v>2026-11-27T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H21" s="183" t="d">
+        <x:v>2026-11-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I21" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J21" s="151" t="str">
+        <x:v>T0067 enquiry identity and contact workflows complete.</x:v>
+      </x:c>
+      <x:c r="K21" s="151" t="str">
+        <x:v>Confirm operating hours, blackout dates, lead time, capacity, reminder channels, cancellation rules, and calendar ownership.</x:v>
+      </x:c>
+      <x:c r="L21" s="151" t="str">
+        <x:v>Planned: deliver user-confirmed visit scheduling with conflict prevention, staff ownership, and complete status history.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="150" t="n">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="B22" s="150" t="str">
+        <x:v>T0070</x:v>
+      </x:c>
+      <x:c r="C22" s="151" t="str">
+        <x:v>Add operational notifications</x:v>
+      </x:c>
+      <x:c r="D22" s="151" t="str">
+        <x:v>Notify authorized users about enquiries, visits, approvals, expired facts, failed AI releases, provider incidents, and security events.</x:v>
+      </x:c>
+      <x:c r="E22" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F22" s="153" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G22" s="183" t="d">
+        <x:v>2026-11-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H22" s="183" t="d">
+        <x:v>2026-12-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I22" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J22" s="151" t="str">
+        <x:v>T0062-T0068 workflow events defined.</x:v>
+      </x:c>
+      <x:c r="K22" s="151" t="str">
+        <x:v>Approve recipients, channels, quiet hours, templates, retry limits, escalation paths, and suppression of sensitive content.</x:v>
+      </x:c>
+      <x:c r="L22" s="151" t="str">
+        <x:v>Planned: provide actionable, permission-aware notifications without exposing private data or creating alert fatigue.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="150" t="n">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B23" s="150" t="str">
+        <x:v>T0071</x:v>
+      </x:c>
+      <x:c r="C23" s="151" t="str">
+        <x:v>Build analytics and reporting</x:v>
+      </x:c>
+      <x:c r="D23" s="151" t="str">
+        <x:v>Create aggregate dashboards for inventory, enquiries, visits, content freshness, AI quality, language use, handoffs, latency, reliability, and approved costs.</x:v>
+      </x:c>
+      <x:c r="E23" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F23" s="153" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G23" s="183" t="d">
+        <x:v>2026-12-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H23" s="183" t="d">
+        <x:v>2026-12-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I23" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J23" s="151" t="str">
+        <x:v>T0067-T0069 operational data and privacy taxonomy available.</x:v>
+      </x:c>
+      <x:c r="K23" s="151" t="str">
+        <x:v>Reports must use approved aggregate measures and avoid raw conversations, audio, contact content, or invasive visitor tracking.</x:v>
+      </x:c>
+      <x:c r="L23" s="151" t="str">
+        <x:v>Planned: deliver role-aware business and AI reporting with metric definitions, filters, and export controls.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="150" t="n">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="B24" s="150" t="str">
+        <x:v>T0072</x:v>
+      </x:c>
+      <x:c r="C24" s="151" t="str">
+        <x:v>Add audit and retention controls</x:v>
+      </x:c>
+      <x:c r="D24" s="151" t="str">
+        <x:v>Record immutable administrative actions and automate approved retention, expiry, deletion, legal hold, and evidence-preservation rules.</x:v>
+      </x:c>
+      <x:c r="E24" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F24" s="153" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G24" s="183" t="d">
+        <x:v>2026-12-04T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H24" s="183" t="d">
+        <x:v>2026-12-05T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I24" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J24" s="151" t="str">
+        <x:v>T0055 policies and all administrative workflows defined.</x:v>
+      </x:c>
+      <x:c r="K24" s="151" t="str">
+        <x:v>Confirm audit visibility, retention periods, deletion exceptions, export approval, and recovery evidence before automation.</x:v>
+      </x:c>
+      <x:c r="L24" s="151" t="str">
+        <x:v>Planned: provide searchable audit history and policy-driven lifecycle controls for sensitive and operational records.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="150" t="n">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="B25" s="150" t="str">
+        <x:v>T0073</x:v>
+      </x:c>
+      <x:c r="C25" s="151" t="str">
+        <x:v>Add backups and recovery</x:v>
+      </x:c>
+      <x:c r="D25" s="151" t="str">
+        <x:v>Implement encrypted backups, restore testing, recovery objectives, service-failure procedures, and database, storage, index, and configuration runbooks.</x:v>
+      </x:c>
+      <x:c r="E25" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F25" s="153" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G25" s="183" t="d">
+        <x:v>2026-12-06T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H25" s="183" t="d">
+        <x:v>2026-12-07T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I25" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J25" s="151" t="str">
+        <x:v>T0057 services and T0071 lifecycle controls complete.</x:v>
+      </x:c>
+      <x:c r="K25" s="151" t="str">
+        <x:v>Approve recovery time and recovery point objectives, backup retention, access ownership, and disaster communication steps.</x:v>
+      </x:c>
+      <x:c r="L25" s="151" t="str">
+        <x:v>Planned: prove recoverability through documented restoration tests rather than backup creation alone.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="150" t="n">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="B26" s="150" t="str">
+        <x:v>T0074</x:v>
+      </x:c>
+      <x:c r="C26" s="151" t="str">
+        <x:v>Harden quality and security</x:v>
+      </x:c>
+      <x:c r="D26" s="151" t="str">
+        <x:v>Complete threat remediation, dependency review, authorization tests, upload security, accessibility, performance, privacy, abuse, and resilience checks.</x:v>
+      </x:c>
+      <x:c r="E26" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F26" s="153" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G26" s="183" t="d">
+        <x:v>2026-12-08T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H26" s="183" t="d">
+        <x:v>2026-12-10T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I26" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J26" s="151" t="str">
+        <x:v>T0059-T0072 features and recovery controls complete.</x:v>
+      </x:c>
+      <x:c r="K26" s="151" t="str">
+        <x:v>All critical or high-severity findings, permission bypasses, privacy defects, accessibility blockers, and data-loss risks block release.</x:v>
+      </x:c>
+      <x:c r="L26" s="151" t="str">
+        <x:v>Planned: produce a signed hardening report with resolved findings, accepted residual risks, and repeatable regression checks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="150" t="n">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="B27" s="150" t="str">
+        <x:v>T0075</x:v>
+      </x:c>
+      <x:c r="C27" s="151" t="str">
+        <x:v>Run integration and UAT</x:v>
+      </x:c>
+      <x:c r="D27" s="151" t="str">
+        <x:v>Test end-to-end owner, content, villa, AI publishing, enquiry, visit, analytics, notification, backup, desktop, and mobile journeys.</x:v>
+      </x:c>
+      <x:c r="E27" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F27" s="153" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="G27" s="183" t="d">
+        <x:v>2026-12-11T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H27" s="183" t="d">
+        <x:v>2026-12-13T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I27" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J27" s="151" t="str">
+        <x:v>T0073 hardening complete and release candidate deployed to an isolated preview.</x:v>
+      </x:c>
+      <x:c r="K27" s="151" t="str">
+        <x:v>Use synthetic non-personal data; define acceptance scenarios, reviewers, evidence, defect severity, and retest requirements before execution.</x:v>
+      </x:c>
+      <x:c r="L27" s="151" t="str">
+        <x:v>Planned: complete integration, browser, migration, recovery, and owner UAT with all release-blocking defects resolved.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="150" t="n">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="B28" s="150" t="str">
+        <x:v>T0076</x:v>
+      </x:c>
+      <x:c r="C28" s="151" t="str">
+        <x:v>Conduct owner pilot and training</x:v>
+      </x:c>
+      <x:c r="D28" s="151" t="str">
+        <x:v>Run controlled daily operations, train the owner, validate support procedures, collect feedback, and confirm operational readiness.</x:v>
+      </x:c>
+      <x:c r="E28" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F28" s="153" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G28" s="183" t="d">
+        <x:v>2026-12-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H28" s="183" t="d">
+        <x:v>2026-12-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I28" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J28" s="151" t="str">
+        <x:v>T0074 UAT accepted.</x:v>
+      </x:c>
+      <x:c r="K28" s="151" t="str">
+        <x:v>AKHIL must confirm training topics, pilot data, support ownership, launch communications, and final acceptance criteria.</x:v>
+      </x:c>
+      <x:c r="L28" s="151" t="str">
+        <x:v>Planned: complete the owner pilot, operating guide, training evidence, support matrix, and formal launch approval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="150" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="B29" s="150" t="str">
+        <x:v>T0077</x:v>
+      </x:c>
+      <x:c r="C29" s="151" t="str">
+        <x:v>Release Phase 3 MVP</x:v>
+      </x:c>
+      <x:c r="D29" s="151" t="str">
+        <x:v>Deploy the exact accepted artifact, run migrations and smoke checks, verify monitoring and backups, promote publicly, and preserve the release version.</x:v>
+      </x:c>
+      <x:c r="E29" s="152" t="str">
+        <x:v>AKHIL</x:v>
+      </x:c>
+      <x:c r="F29" s="153" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G29" s="183" t="d">
+        <x:v>2026-12-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H29" s="183" t="d">
+        <x:v>2026-12-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I29" s="150" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="J29" s="151" t="str">
+        <x:v>T0075 accepted with owner approval; production change window and rollback readiness confirmed.</x:v>
+      </x:c>
+      <x:c r="K29" s="151" t="str">
+        <x:v>Release requires migration backup, tested rollback, incident ownership, production limits, privacy checks, launch approval, and post-release monitoring.</x:v>
+      </x:c>
+      <x:c r="L29" s="151" t="str">
+        <x:v>Planned: release the secure owner operations platform only after every Phase 3 gate passes and preserve the resulting stable version.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="155"/>
+      <x:c r="B30" s="155"/>
+      <x:c r="C30" s="156"/>
+      <x:c r="D30" s="156"/>
+      <x:c r="E30" s="157"/>
+      <x:c r="F30" s="158"/>
+      <x:c r="G30" s="184"/>
+      <x:c r="H30" s="184"/>
+      <x:c r="I30" s="155"/>
+      <x:c r="J30" s="156"/>
+      <x:c r="K30" s="156"/>
+      <x:c r="L30" s="156"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:L1"/>
+    <x:mergeCell ref="A2:L2"/>
+    <x:mergeCell ref="A3:L3"/>
+  </x:mergeCells>
+  <x:dataValidations count="2">
+    <x:dataValidation type="list" sqref="E6:E29">
+      <x:formula1>"AKHIL"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="I6:I29">
+      <x:formula1>"Not Started,Planned,In Progress,On Hold,Completed,Blocked"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4de6ffaa7b54636"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Define secure Phase 3 architecture
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R273578b0ead34caa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R29ec8333793540ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R548105d511134bf1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Racdadb2e607f4740"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R081f9d39377a4af6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R35c0fc6b56564d13"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3 MVP" sheetId="7" r:id="Ra0e8672437fe4d1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R762f76ec96ca493d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R157a247e846943e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R08502e7ec197407d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R9a4d476d91754de2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R9fdf8015f28847ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R385e38de9fbb4169"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3 MVP" sheetId="7" r:id="R72ffebed471c443e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3226,7 +3226,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b8384a7a18b4f8e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd64ed43871f4f8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4323,7 +4323,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3acd7cfa8356486c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3476a47142914383"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5101,7 +5101,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfec130c011cc4d80"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87824df359b94eca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6078,7 +6078,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16b0b94415ec432a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10261ac4a9fd4124"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6365,25 +6365,25 @@
         <x:v>AKHIL</x:v>
       </x:c>
       <x:c r="F8" s="153" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G8" s="183" t="d">
-        <x:v>2026-10-28T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="H8" s="183" t="d">
-        <x:v>2026-10-29T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I8" s="150" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J8" s="151" t="str">
-        <x:v>T0054-T0055 approved.</x:v>
+        <x:v>Completed after T0054-T0055 approval. T0057 may proceed after owner authorization.</x:v>
       </x:c>
       <x:c r="K8" s="151" t="str">
-        <x:v>Select managed services only after security, cost, portability, and recovery requirements are reviewed.</x:v>
+        <x:v>Resolved: Vercel, Supabase, and Resend are selected conditionally. Exact regions, plans, limits, costs, and provisioning remain in T0057.</x:v>
       </x:c>
       <x:c r="L8" s="151" t="str">
-        <x:v>Planned: produce the reviewed architecture, trust boundaries, threat model, service choices, and failure strategy.</x:v>
+        <x:v>Completed: approved secure architecture, trust boundaries, STRIDE threat model, managed-service decision, recovery objectives, and failure strategy are documented in docs/phase-3/secure-architecture.md, threat-model.md, and service-decision-record.md.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -7214,7 +7214,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4de6ffaa7b54636"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3981785bfd0841c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Configure isolated database and storage
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R762f76ec96ca493d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R157a247e846943e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R08502e7ec197407d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="R9a4d476d91754de2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R9fdf8015f28847ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R385e38de9fbb4169"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3 MVP" sheetId="7" r:id="R72ffebed471c443e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R75c3fbcd5cd2403a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R95e8d7ed59c44c5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R5987aa0c6d694739"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rd99349e0f6d6479c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R5311a4b0115f479d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R682c64bde3824a82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3 MVP" sheetId="7" r:id="R6ccf10951b7742e1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1420,7 +1420,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="121" t="str">
-        <x:v>Version 1.0.0 is publicly released and preserved. Phase 3 is planned as a secure owner operations platform; implementation remains paused until AKHIL explicitly authorizes it.</x:v>
+        <x:v>Version 1.0.0 is publicly released and preserved. Phase 3 implementation is active under AKHIL's approval; T0057 database and storage configuration is complete and T0058 is next.</x:v>
       </x:c>
       <x:c r="B2" s="120"/>
       <x:c r="C2" s="120"/>
@@ -3226,7 +3226,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd64ed43871f4f8f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reca1166c42e24e6a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4323,7 +4323,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3476a47142914383"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89cbf8854f6d4fdb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5101,7 +5101,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R87824df359b94eca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d0a971867d04045"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6078,7 +6078,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10261ac4a9fd4124"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83e91b9b00204c9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6406,22 +6406,22 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="G9" s="183" t="d">
-        <x:v>2026-10-30T00:00:00.000Z</x:v>
+        <x:v>2026-10-24T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="H9" s="183" t="d">
-        <x:v>2026-10-31T00:00:00.000Z</x:v>
+        <x:v>2026-10-25T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I9" s="150" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J9" s="151" t="str">
-        <x:v>T0056 architecture approved.</x:v>
+        <x:v>Resolved: T0056 architecture approved; separate preview and production projects and environment scopes are active.</x:v>
       </x:c>
       <x:c r="K9" s="151" t="str">
-        <x:v>Confirm region, budget, data residency, storage limits, and separation between public assets and protected documents.</x:v>
+        <x:v>Resolved: Mumbai selected for both data projects and application functions. USD 0 projects are accepted for initial implementation; verified recovery remains a release gate before real personal data.</x:v>
       </x:c>
       <x:c r="L9" s="151" t="str">
-        <x:v>Planned: configure environment-separated database and storage services without exposing administrative credentials to the browser.</x:v>
+        <x:v>Completed: provisioned isolated Mumbai preview and production projects, verified four bucket records in each, scoped browser-safe Vercel configuration by environment, recorded the Free-plan recovery gate, and passed automated configuration plus hosted security/performance advisor checks. Local Docker smoke test is the T0058 entry check because the installed engine did not become responsive during this run.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -7214,7 +7214,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3981785bfd0841c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53e5ff9a70824c41"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Implement Phase 3 data schema and migrations
</commit_message>
<xml_diff>
--- a/AI-Driven-Gated-Community-Tracker.xlsx
+++ b/AI-Driven-Gated-Community-Tracker.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R75c3fbcd5cd2403a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R95e8d7ed59c44c5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="R5987aa0c6d694739"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Rd99349e0f6d6479c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="R5311a4b0115f479d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R682c64bde3824a82"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3 MVP" sheetId="7" r:id="R6ccf10951b7742e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R37d45e85b18e4973"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 1 MVP" sheetId="2" r:id="R681e5d26e5174a1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 2 MVP" sheetId="3" r:id="Rad9f6cef12ab414e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code Review Guidelines" sheetId="4" r:id="Re29db0e31cf84b9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requirements" sheetId="5" r:id="Rde5209b237fc4449"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" r:id="R274f988eeb1448d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase 3 MVP" sheetId="7" r:id="Rc9c67d4b66114a7a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1420,7 +1420,7 @@
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="121" t="str">
-        <x:v>Version 1.0.0 is publicly released and preserved. Phase 3 implementation is active under AKHIL's approval; T0057 database and storage configuration is complete and T0058 is next.</x:v>
+        <x:v>Version 1.0.0 is publicly released and preserved. Phase 3 implementation is active under AKHIL's approval; T0058 schema and migrations are complete and T0059 authentication is next.</x:v>
       </x:c>
       <x:c r="B2" s="120"/>
       <x:c r="C2" s="120"/>
@@ -3226,7 +3226,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reca1166c42e24e6a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R798e2df8ab004436"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4323,7 +4323,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89cbf8854f6d4fdb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd8483629758e4f1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5101,7 +5101,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d0a971867d04045"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41841faff8224ff2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6078,7 +6078,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83e91b9b00204c9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf954372d5aa54ff8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6441,25 +6441,25 @@
         <x:v>AKHIL</x:v>
       </x:c>
       <x:c r="F10" s="153" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="G10" s="183" t="d">
-        <x:v>2026-11-01T00:00:00.000Z</x:v>
+        <x:v>2026-10-25T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="H10" s="183" t="d">
-        <x:v>2026-11-02T00:00:00.000Z</x:v>
+        <x:v>2026-10-25T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I10" s="150" t="str">
-        <x:v>Planned</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="J10" s="151" t="str">
-        <x:v>T0057 services configured.</x:v>
+        <x:v>Resolved: T0057 services configured. The local Docker entry check was unavailable, so the isolated Preview environment was used first for transactional migration verification before Production.</x:v>
       </x:c>
       <x:c r="K10" s="151" t="str">
-        <x:v>Define stable identifiers, lifecycle states, ownership, timestamps, deletion rules, and migration rollback requirements.</x:v>
+        <x:v>Resolved: stable UUID identifiers, constrained lifecycle states, ownership references, UTC timestamps, retention fields, append-only audits, synthetic seeds, and forward-only rollback rules are documented and enforced.</x:v>
       </x:c>
       <x:c r="L10" s="151" t="str">
-        <x:v>Planned: deliver reviewed schemas, constraints, seed strategy, migrations, and rollback-tested development data.</x:v>
+        <x:v>Completed: delivered two versioned migrations for 16 private canonical tables, 16 forced-RLS tables, 16 explicit deny policies, 67 indexes, synthetic seeds, pgTAP and application contract tests, rollback guidance, and identical Preview-to-Production promotion. Constraint probes passed; both environments have zero browser grants and zero security advisor findings.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -7214,7 +7214,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53e5ff9a70824c41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93f3525260684919"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>